<commit_message>
Hop totaal gewicht: A67:A70 (soort 1-4) + I67:I70 (soort 5-8) apart en robuust
Klopte niet met de layout: het origineel heeft twee losse kolomparen
(A/E = eerste 4 unieke soorten, I/M = volgende 4), niet één. Ook gevonden
waarom tabel 2 stukging: die hing af van R66:R73-hulpcellen die per ongeluk
zijn meegeveegd bij het opschonen van kolom Q en verder.

Beide tabellen nu volledig onafhankelijk van elkaar en van enige
hulpkolom: elke cel is een simpele INDEX(UNIQUE(FILTER(...)),N)-formule
die zijn eigen Nde unieke waarde uit A43:A63 pakt (N=1..4 voor tabel 1,
N=5..8 voor tabel 2). Geen array-formule-declaratie nodig (INDEX met een
vaste positie is een gewone formule), geen zelf-refererende keten meer die
kan breken. E67:E70/M67:M70 (de SUMIF-optelling) ongewijzigd, blijven live.
</commit_message>
<xml_diff>
--- a/batchrapport-generator/Batchrapport_sjabloon.xlsx
+++ b/batchrapport-generator/Batchrapport_sjabloon.xlsx
@@ -12283,7 +12283,7 @@
     </row>
     <row r="67" ht="15" customFormat="1" customHeight="1" s="1221">
       <c r="A67" s="1277">
-        <f>IFERROR(INDEX(A$43:A$63,MATCH(FALSE(),ISNUMBER(MATCH(A$43:A$63,A64:A66,0)),0)),"")</f>
+        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),1),"")</f>
         <v/>
       </c>
       <c r="B67" s="1278" t="n"/>
@@ -12297,7 +12297,7 @@
       <c r="G67" s="1223" t="n"/>
       <c r="H67" s="1224" t="n"/>
       <c r="I67" s="1281">
-        <f t="array" ref="I67:I70">IFERROR(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),"")</f>
+        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),5),"")</f>
         <v/>
       </c>
       <c r="J67" s="1223" t="n"/>
@@ -12318,7 +12318,7 @@
     </row>
     <row r="68" ht="15" customFormat="1" customHeight="1" s="1221">
       <c r="A68" s="1282">
-        <f>IFERROR(INDEX(A$44:A$63,MATCH(FALSE(),ISNUMBER(MATCH(A$44:A$63,$A$64:A67,0)),0)),"")</f>
+        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),2),"")</f>
         <v/>
       </c>
       <c r="B68" s="1177" t="n"/>
@@ -12331,7 +12331,10 @@
       <c r="F68" s="1245" t="n"/>
       <c r="G68" s="1245" t="n"/>
       <c r="H68" s="1227" t="n"/>
-      <c r="I68" s="1282" t="n"/>
+      <c r="I68" s="1282">
+        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),6),"")</f>
+        <v/>
+      </c>
       <c r="J68" s="1177" t="n"/>
       <c r="K68" s="1177" t="n"/>
       <c r="L68" s="1178" t="n"/>
@@ -12350,7 +12353,7 @@
     </row>
     <row r="69" ht="15" customFormat="1" customHeight="1" s="1221">
       <c r="A69" s="1282">
-        <f>IFERROR(INDEX(A$45:A$63,MATCH(FALSE(),ISNUMBER(MATCH(A$45:A$63,$A$64:A68,0)),0)),"")</f>
+        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),3),"")</f>
         <v/>
       </c>
       <c r="B69" s="1177" t="n"/>
@@ -12363,7 +12366,10 @@
       <c r="F69" s="1245" t="n"/>
       <c r="G69" s="1245" t="n"/>
       <c r="H69" s="1227" t="n"/>
-      <c r="I69" s="1282" t="n"/>
+      <c r="I69" s="1282">
+        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),7),"")</f>
+        <v/>
+      </c>
       <c r="J69" s="1177" t="n"/>
       <c r="K69" s="1177" t="n"/>
       <c r="L69" s="1178" t="n"/>
@@ -12382,7 +12388,7 @@
     </row>
     <row r="70" ht="15" customFormat="1" customHeight="1" s="1221">
       <c r="A70" s="1283">
-        <f>IFERROR(INDEX(A$45:A$63,MATCH(FALSE(),ISNUMBER(MATCH(A$45:A$63,$A$64:A69,0)),0)),"")</f>
+        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),4),"")</f>
         <v/>
       </c>
       <c r="B70" s="1198" t="n"/>
@@ -12395,7 +12401,10 @@
       <c r="F70" s="1198" t="n"/>
       <c r="G70" s="1198" t="n"/>
       <c r="H70" s="1199" t="n"/>
-      <c r="I70" s="1283" t="n"/>
+      <c r="I70" s="1283">
+        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),8),"")</f>
+        <v/>
+      </c>
       <c r="J70" s="1198" t="n"/>
       <c r="K70" s="1198" t="n"/>
       <c r="L70" s="1199" t="n"/>

</xml_diff>

<commit_message>
Batchrapport: Hop totaal gewicht sjabloon uitgebreid naar 12 unieke soorten (2x6)
</commit_message>
<xml_diff>
--- a/batchrapport-generator/Batchrapport_sjabloon.xlsx
+++ b/batchrapport-generator/Batchrapport_sjabloon.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xleta.ROUND" hidden="1" function="0" vbProcedure="0">#NAME?</definedName>
     <definedName name="_xleta.ROUNDUP" hidden="1" function="0" vbProcedure="0">#NAME?</definedName>
     <definedName name="_xleta.TYPE" hidden="1" function="0" vbProcedure="0">#NAME?</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Recept-voorblad'!$A$1:$P$105</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Recept-voorblad'!$A$1:$P$107</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -10062,7 +10062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AG107"/>
+  <dimension ref="A1:AG109"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.00390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4.5" customWidth="1" style="1069" min="1" max="2"/>
@@ -12284,28 +12284,24 @@
     <row r="67" ht="15" customFormat="1" customHeight="1" s="1221">
       <c r="A67" s="1277">
         <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),1),"")</f>
-        <v/>
       </c>
       <c r="B67" s="1278" t="n"/>
       <c r="C67" s="1278" t="n"/>
       <c r="D67" s="1279" t="n"/>
       <c r="E67" s="1280">
         <f>IF(A67="","",SUMIF($A$43:$A$63,A67,$P$43:$P$63))</f>
-        <v/>
       </c>
       <c r="F67" s="1223" t="n"/>
       <c r="G67" s="1223" t="n"/>
       <c r="H67" s="1224" t="n"/>
       <c r="I67" s="1281">
-        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),5),"")</f>
-        <v/>
+        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),7),"")</f>
       </c>
       <c r="J67" s="1223" t="n"/>
       <c r="K67" s="1223" t="n"/>
       <c r="L67" s="1224" t="n"/>
       <c r="M67" s="1243">
         <f>IF(I67="","",SUMIF($A$43:$A$63,I67,$P$43:$P$63))</f>
-        <v/>
       </c>
       <c r="N67" s="1198" t="n"/>
       <c r="O67" s="1198" t="n"/>
@@ -12319,28 +12315,24 @@
     <row r="68" ht="15" customFormat="1" customHeight="1" s="1221">
       <c r="A68" s="1282">
         <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),2),"")</f>
-        <v/>
       </c>
       <c r="B68" s="1177" t="n"/>
       <c r="C68" s="1177" t="n"/>
       <c r="D68" s="1178" t="n"/>
       <c r="E68" s="1232">
-        <f>IF(A68="","",SUMIF($A$43:$A$64,A68,$P$43:$P$64))</f>
-        <v/>
+        <f>IF(A68="","",SUMIF($A$43:$A$63,A68,$P$43:$P$63))</f>
       </c>
       <c r="F68" s="1245" t="n"/>
       <c r="G68" s="1245" t="n"/>
       <c r="H68" s="1227" t="n"/>
       <c r="I68" s="1282">
-        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),6),"")</f>
-        <v/>
+        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),8),"")</f>
       </c>
       <c r="J68" s="1177" t="n"/>
       <c r="K68" s="1177" t="n"/>
       <c r="L68" s="1178" t="n"/>
       <c r="M68" s="1232">
         <f>IF(I68="","",SUMIF($A$43:$A$63,I68,$P$43:$P$63))</f>
-        <v/>
       </c>
       <c r="N68" s="1245" t="n"/>
       <c r="O68" s="1245" t="n"/>
@@ -12354,28 +12346,24 @@
     <row r="69" ht="15" customFormat="1" customHeight="1" s="1221">
       <c r="A69" s="1282">
         <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),3),"")</f>
-        <v/>
       </c>
       <c r="B69" s="1177" t="n"/>
       <c r="C69" s="1177" t="n"/>
       <c r="D69" s="1178" t="n"/>
       <c r="E69" s="1232">
         <f>IF(A69="","",SUMIF($A$43:$A$63,A69,$P$43:$P$63))</f>
-        <v/>
       </c>
       <c r="F69" s="1245" t="n"/>
       <c r="G69" s="1245" t="n"/>
       <c r="H69" s="1227" t="n"/>
       <c r="I69" s="1282">
-        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),7),"")</f>
-        <v/>
+        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),9),"")</f>
       </c>
       <c r="J69" s="1177" t="n"/>
       <c r="K69" s="1177" t="n"/>
       <c r="L69" s="1178" t="n"/>
       <c r="M69" s="1232">
         <f>IF(I69="","",SUMIF($A$43:$A$63,I69,$P$43:$P$63))</f>
-        <v/>
       </c>
       <c r="N69" s="1245" t="n"/>
       <c r="O69" s="1245" t="n"/>
@@ -12389,28 +12377,24 @@
     <row r="70" ht="15" customFormat="1" customHeight="1" s="1221">
       <c r="A70" s="1283">
         <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),4),"")</f>
-        <v/>
       </c>
       <c r="B70" s="1198" t="n"/>
       <c r="C70" s="1198" t="n"/>
       <c r="D70" s="1199" t="n"/>
       <c r="E70" s="1243">
         <f>IF(A70="","",SUMIF($A$43:$A$63,A70,$P$43:$P$63))</f>
-        <v/>
       </c>
       <c r="F70" s="1198" t="n"/>
       <c r="G70" s="1198" t="n"/>
       <c r="H70" s="1199" t="n"/>
       <c r="I70" s="1283">
-        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),8),"")</f>
-        <v/>
+        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),10),"")</f>
       </c>
       <c r="J70" s="1198" t="n"/>
       <c r="K70" s="1198" t="n"/>
       <c r="L70" s="1199" t="n"/>
       <c r="M70" s="1243">
         <f>IF(I70="","",SUMIF($A$43:$A$63,I70,$P$43:$P$63))</f>
-        <v/>
       </c>
       <c r="N70" s="1198" t="n"/>
       <c r="O70" s="1198" t="n"/>
@@ -12421,27 +12405,31 @@
       <c r="T70" s="1139" t="n"/>
       <c r="U70" s="1188" t="n"/>
     </row>
-    <row r="71" ht="18.75" customFormat="1" customHeight="1" s="1221">
-      <c r="A71" s="1284" t="inlineStr">
-        <is>
-          <t>Additions Brewers</t>
-        </is>
-      </c>
-      <c r="B71" s="1080" t="n"/>
-      <c r="C71" s="1080" t="n"/>
-      <c r="D71" s="1080" t="n"/>
-      <c r="E71" s="1080" t="n"/>
-      <c r="F71" s="1080" t="n"/>
-      <c r="G71" s="1080" t="n"/>
-      <c r="H71" s="1080" t="n"/>
-      <c r="I71" s="1080" t="n"/>
-      <c r="J71" s="1080" t="n"/>
-      <c r="K71" s="1080" t="n"/>
-      <c r="L71" s="1080" t="n"/>
-      <c r="M71" s="1080" t="n"/>
-      <c r="N71" s="1080" t="n"/>
-      <c r="O71" s="1080" t="n"/>
-      <c r="P71" s="1081" t="n"/>
+    <row r="71" ht="15" customFormat="1" customHeight="1" s="1221">
+      <c r="A71" s="1283">
+        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),5),"")</f>
+      </c>
+      <c r="B71" s="1198" t="n"/>
+      <c r="C71" s="1198" t="n"/>
+      <c r="D71" s="1199" t="n"/>
+      <c r="E71" s="1243">
+        <f>IF(A71="","",SUMIF($A$43:$A$63,A71,$P$43:$P$63))</f>
+      </c>
+      <c r="F71" s="1198" t="n"/>
+      <c r="G71" s="1198" t="n"/>
+      <c r="H71" s="1199" t="n"/>
+      <c r="I71" s="1283">
+        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),11),"")</f>
+      </c>
+      <c r="J71" s="1198" t="n"/>
+      <c r="K71" s="1198" t="n"/>
+      <c r="L71" s="1199" t="n"/>
+      <c r="M71" s="1243">
+        <f>IF(I71="","",SUMIF($A$43:$A$63,I71,$P$43:$P$63))</f>
+      </c>
+      <c r="N71" s="1198" t="n"/>
+      <c r="O71" s="1198" t="n"/>
+      <c r="P71" s="1199" t="n"/>
       <c r="Q71" s="1138" t="n"/>
       <c r="R71" s="1139" t="n"/>
       <c r="S71" s="1139" t="n"/>
@@ -12449,61 +12437,57 @@
       <c r="U71" s="1188" t="n"/>
     </row>
     <row r="72" ht="15" customFormat="1" customHeight="1" s="1221">
-      <c r="A72" s="1285" t="inlineStr">
-        <is>
-          <t>Soort</t>
-        </is>
-      </c>
-      <c r="B72" s="1114" t="n"/>
-      <c r="C72" s="1114" t="n"/>
-      <c r="D72" s="1115" t="n"/>
-      <c r="E72" s="1286" t="inlineStr">
-        <is>
-          <t>Hoeveelheid</t>
-        </is>
-      </c>
-      <c r="F72" s="1114" t="n"/>
-      <c r="G72" s="1114" t="n"/>
-      <c r="H72" s="1114" t="n"/>
-      <c r="I72" s="1287" t="inlineStr">
-        <is>
-          <t>Wanneer</t>
-        </is>
-      </c>
-      <c r="J72" s="1114" t="n"/>
-      <c r="K72" s="1115" t="n"/>
-      <c r="L72" s="1288" t="inlineStr">
-        <is>
-          <t>Lotnummer</t>
-        </is>
-      </c>
-      <c r="M72" s="1080" t="n"/>
-      <c r="N72" s="1080" t="n"/>
-      <c r="O72" s="1080" t="n"/>
-      <c r="P72" s="1081" t="n"/>
+      <c r="A72" s="1283">
+        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),6),"")</f>
+      </c>
+      <c r="B72" s="1198" t="n"/>
+      <c r="C72" s="1198" t="n"/>
+      <c r="D72" s="1199" t="n"/>
+      <c r="E72" s="1243">
+        <f>IF(A72="","",SUMIF($A$43:$A$63,A72,$P$43:$P$63))</f>
+      </c>
+      <c r="F72" s="1198" t="n"/>
+      <c r="G72" s="1198" t="n"/>
+      <c r="H72" s="1199" t="n"/>
+      <c r="I72" s="1283">
+        <f>IFERROR(INDEX(_xlfn.UNIQUE(_xlfn._xlws.FILTER($A$43:$A$63,$A$43:$A$63&lt;&gt;"")),12),"")</f>
+      </c>
+      <c r="J72" s="1198" t="n"/>
+      <c r="K72" s="1198" t="n"/>
+      <c r="L72" s="1199" t="n"/>
+      <c r="M72" s="1243">
+        <f>IF(I72="","",SUMIF($A$43:$A$63,I72,$P$43:$P$63))</f>
+      </c>
+      <c r="N72" s="1198" t="n"/>
+      <c r="O72" s="1198" t="n"/>
+      <c r="P72" s="1199" t="n"/>
       <c r="Q72" s="1138" t="n"/>
       <c r="R72" s="1139" t="n"/>
       <c r="S72" s="1139" t="n"/>
       <c r="T72" s="1139" t="n"/>
       <c r="U72" s="1188" t="n"/>
     </row>
-    <row r="73" ht="17.25" customFormat="1" customHeight="1" s="1221">
-      <c r="A73" s="1289" t="n"/>
-      <c r="B73" s="1177" t="n"/>
-      <c r="C73" s="1177" t="n"/>
-      <c r="D73" s="1178" t="n"/>
-      <c r="E73" s="1290" t="n"/>
-      <c r="F73" s="1177" t="n"/>
-      <c r="G73" s="1177" t="n"/>
-      <c r="H73" s="1177" t="n"/>
-      <c r="I73" s="1291" t="n"/>
-      <c r="J73" s="1223" t="n"/>
-      <c r="K73" s="1224" t="n"/>
-      <c r="L73" s="1292" t="n"/>
-      <c r="M73" s="1177" t="n"/>
-      <c r="N73" s="1177" t="n"/>
-      <c r="O73" s="1177" t="n"/>
-      <c r="P73" s="1178" t="n"/>
+    <row r="73" ht="18.75" customFormat="1" customHeight="1" s="1221">
+      <c r="A73" s="1284" t="inlineStr">
+        <is>
+          <t>Additions Brewers</t>
+        </is>
+      </c>
+      <c r="B73" s="1080" t="n"/>
+      <c r="C73" s="1080" t="n"/>
+      <c r="D73" s="1080" t="n"/>
+      <c r="E73" s="1080" t="n"/>
+      <c r="F73" s="1080" t="n"/>
+      <c r="G73" s="1080" t="n"/>
+      <c r="H73" s="1080" t="n"/>
+      <c r="I73" s="1080" t="n"/>
+      <c r="J73" s="1080" t="n"/>
+      <c r="K73" s="1080" t="n"/>
+      <c r="L73" s="1080" t="n"/>
+      <c r="M73" s="1080" t="n"/>
+      <c r="N73" s="1080" t="n"/>
+      <c r="O73" s="1080" t="n"/>
+      <c r="P73" s="1081" t="n"/>
       <c r="Q73" s="1138" t="n"/>
       <c r="R73" s="1139" t="n"/>
       <c r="S73" s="1139" t="n"/>
@@ -12511,40 +12495,56 @@
       <c r="U73" s="1188" t="n"/>
     </row>
     <row r="74" ht="15" customFormat="1" customHeight="1" s="1221">
-      <c r="A74" s="1289" t="n"/>
-      <c r="B74" s="1177" t="n"/>
-      <c r="C74" s="1177" t="n"/>
-      <c r="D74" s="1178" t="n"/>
-      <c r="E74" s="1293" t="n"/>
-      <c r="F74" s="1177" t="n"/>
-      <c r="G74" s="1177" t="n"/>
-      <c r="H74" s="1178" t="n"/>
-      <c r="I74" s="1289" t="n"/>
-      <c r="J74" s="1177" t="n"/>
-      <c r="K74" s="1178" t="n"/>
-      <c r="L74" s="1292" t="n"/>
-      <c r="M74" s="1177" t="n"/>
-      <c r="N74" s="1177" t="n"/>
-      <c r="O74" s="1177" t="n"/>
-      <c r="P74" s="1178" t="n"/>
+      <c r="A74" s="1285" t="inlineStr">
+        <is>
+          <t>Soort</t>
+        </is>
+      </c>
+      <c r="B74" s="1114" t="n"/>
+      <c r="C74" s="1114" t="n"/>
+      <c r="D74" s="1115" t="n"/>
+      <c r="E74" s="1286" t="inlineStr">
+        <is>
+          <t>Hoeveelheid</t>
+        </is>
+      </c>
+      <c r="F74" s="1114" t="n"/>
+      <c r="G74" s="1114" t="n"/>
+      <c r="H74" s="1114" t="n"/>
+      <c r="I74" s="1287" t="inlineStr">
+        <is>
+          <t>Wanneer</t>
+        </is>
+      </c>
+      <c r="J74" s="1114" t="n"/>
+      <c r="K74" s="1115" t="n"/>
+      <c r="L74" s="1288" t="inlineStr">
+        <is>
+          <t>Lotnummer</t>
+        </is>
+      </c>
+      <c r="M74" s="1080" t="n"/>
+      <c r="N74" s="1080" t="n"/>
+      <c r="O74" s="1080" t="n"/>
+      <c r="P74" s="1081" t="n"/>
       <c r="Q74" s="1138" t="n"/>
       <c r="R74" s="1139" t="n"/>
       <c r="S74" s="1139" t="n"/>
       <c r="T74" s="1139" t="n"/>
       <c r="U74" s="1188" t="n"/>
     </row>
-    <row r="75" ht="15" customFormat="1" customHeight="1" s="1221">
+    <row r="75" ht="17.25" customFormat="1" customHeight="1" s="1221">
       <c r="A75" s="1289" t="n"/>
       <c r="B75" s="1177" t="n"/>
       <c r="C75" s="1177" t="n"/>
       <c r="D75" s="1178" t="n"/>
-      <c r="E75" s="1293" t="n"/>
+      <c r="E75" s="1290" t="n"/>
       <c r="F75" s="1177" t="n"/>
       <c r="G75" s="1177" t="n"/>
-      <c r="H75" s="1178" t="n"/>
-      <c r="I75" s="1289" t="n"/>
-      <c r="J75" s="1177" t="n"/>
-      <c r="K75" s="1178" t="n"/>
+      <c r="H75" s="1177" t="n"/>
+      <c r="I75" s="1291" t="n"/>
+      <c r="J75" s="1223" t="n"/>
+      <c r="K75" s="1224" t="n"/>
       <c r="L75" s="1292" t="n"/>
       <c r="M75" s="1177" t="n"/>
       <c r="N75" s="1177" t="n"/>
@@ -12584,7 +12584,7 @@
       <c r="B77" s="1177" t="n"/>
       <c r="C77" s="1177" t="n"/>
       <c r="D77" s="1178" t="n"/>
-      <c r="E77" s="1294" t="n"/>
+      <c r="E77" s="1293" t="n"/>
       <c r="F77" s="1177" t="n"/>
       <c r="G77" s="1177" t="n"/>
       <c r="H77" s="1178" t="n"/>
@@ -12630,7 +12630,7 @@
       <c r="B79" s="1177" t="n"/>
       <c r="C79" s="1177" t="n"/>
       <c r="D79" s="1178" t="n"/>
-      <c r="E79" s="1293" t="n"/>
+      <c r="E79" s="1294" t="n"/>
       <c r="F79" s="1177" t="n"/>
       <c r="G79" s="1177" t="n"/>
       <c r="H79" s="1178" t="n"/>
@@ -12699,10 +12699,10 @@
       <c r="B82" s="1177" t="n"/>
       <c r="C82" s="1177" t="n"/>
       <c r="D82" s="1178" t="n"/>
-      <c r="E82" s="1295" t="n"/>
-      <c r="F82" s="1198" t="n"/>
-      <c r="G82" s="1198" t="n"/>
-      <c r="H82" s="1199" t="n"/>
+      <c r="E82" s="1293" t="n"/>
+      <c r="F82" s="1177" t="n"/>
+      <c r="G82" s="1177" t="n"/>
+      <c r="H82" s="1178" t="n"/>
       <c r="I82" s="1289" t="n"/>
       <c r="J82" s="1177" t="n"/>
       <c r="K82" s="1178" t="n"/>
@@ -12717,27 +12717,23 @@
       <c r="T82" s="1139" t="n"/>
       <c r="U82" s="1188" t="n"/>
     </row>
-    <row r="83" ht="15.75" customFormat="1" customHeight="1" s="1221">
-      <c r="A83" s="1215" t="inlineStr">
-        <is>
-          <t>Dry yeast</t>
-        </is>
-      </c>
-      <c r="B83" s="1114" t="n"/>
-      <c r="C83" s="1114" t="n"/>
-      <c r="D83" s="1114" t="n"/>
-      <c r="E83" s="1114" t="n"/>
-      <c r="F83" s="1114" t="n"/>
-      <c r="G83" s="1114" t="n"/>
-      <c r="H83" s="1114" t="n"/>
-      <c r="I83" s="1114" t="n"/>
-      <c r="J83" s="1114" t="n"/>
-      <c r="K83" s="1114" t="n"/>
-      <c r="L83" s="1114" t="n"/>
-      <c r="M83" s="1114" t="n"/>
-      <c r="N83" s="1114" t="n"/>
-      <c r="O83" s="1114" t="n"/>
-      <c r="P83" s="1115" t="n"/>
+    <row r="83" ht="15" customFormat="1" customHeight="1" s="1221">
+      <c r="A83" s="1289" t="n"/>
+      <c r="B83" s="1177" t="n"/>
+      <c r="C83" s="1177" t="n"/>
+      <c r="D83" s="1178" t="n"/>
+      <c r="E83" s="1293" t="n"/>
+      <c r="F83" s="1177" t="n"/>
+      <c r="G83" s="1177" t="n"/>
+      <c r="H83" s="1178" t="n"/>
+      <c r="I83" s="1289" t="n"/>
+      <c r="J83" s="1177" t="n"/>
+      <c r="K83" s="1178" t="n"/>
+      <c r="L83" s="1292" t="n"/>
+      <c r="M83" s="1177" t="n"/>
+      <c r="N83" s="1177" t="n"/>
+      <c r="O83" s="1177" t="n"/>
+      <c r="P83" s="1178" t="n"/>
       <c r="Q83" s="1138" t="n"/>
       <c r="R83" s="1139" t="n"/>
       <c r="S83" s="1139" t="n"/>
@@ -12745,67 +12741,49 @@
       <c r="U83" s="1188" t="n"/>
     </row>
     <row r="84" ht="15" customFormat="1" customHeight="1" s="1221">
-      <c r="A84" s="1296" t="inlineStr">
-        <is>
-          <t>Soort</t>
-        </is>
-      </c>
-      <c r="B84" s="1114" t="n"/>
-      <c r="C84" s="1114" t="n"/>
-      <c r="D84" s="1114" t="n"/>
-      <c r="E84" s="1114" t="n"/>
-      <c r="F84" s="1297" t="inlineStr">
-        <is>
-          <t>Brews/1st day</t>
-        </is>
-      </c>
-      <c r="G84" s="1298" t="inlineStr">
-        <is>
-          <t>Hoeveelheid per batch</t>
-        </is>
-      </c>
-      <c r="H84" s="1114" t="n"/>
-      <c r="I84" s="1114" t="n"/>
-      <c r="J84" s="1114" t="n"/>
-      <c r="K84" s="1115" t="n"/>
-      <c r="L84" s="1299" t="inlineStr">
-        <is>
-          <t>Lotnummer</t>
-        </is>
-      </c>
-      <c r="M84" s="1080" t="n"/>
-      <c r="N84" s="1080" t="n"/>
-      <c r="O84" s="1080" t="n"/>
-      <c r="P84" s="1081" t="n"/>
+      <c r="A84" s="1289" t="n"/>
+      <c r="B84" s="1177" t="n"/>
+      <c r="C84" s="1177" t="n"/>
+      <c r="D84" s="1178" t="n"/>
+      <c r="E84" s="1295" t="n"/>
+      <c r="F84" s="1198" t="n"/>
+      <c r="G84" s="1198" t="n"/>
+      <c r="H84" s="1199" t="n"/>
+      <c r="I84" s="1289" t="n"/>
+      <c r="J84" s="1177" t="n"/>
+      <c r="K84" s="1178" t="n"/>
+      <c r="L84" s="1292" t="n"/>
+      <c r="M84" s="1177" t="n"/>
+      <c r="N84" s="1177" t="n"/>
+      <c r="O84" s="1177" t="n"/>
+      <c r="P84" s="1178" t="n"/>
       <c r="Q84" s="1138" t="n"/>
       <c r="R84" s="1139" t="n"/>
       <c r="S84" s="1139" t="n"/>
       <c r="T84" s="1139" t="n"/>
       <c r="U84" s="1188" t="n"/>
     </row>
-    <row r="85" ht="15" customFormat="1" customHeight="1" s="1221">
-      <c r="A85" s="1300" t="n"/>
-      <c r="B85" s="1223" t="n"/>
-      <c r="C85" s="1223" t="n"/>
-      <c r="D85" s="1223" t="n"/>
-      <c r="E85" s="1223" t="n"/>
-      <c r="F85" s="1301" t="n">
-        <v>1</v>
-      </c>
-      <c r="G85" s="1302" t="n"/>
-      <c r="H85" s="1223" t="n"/>
-      <c r="I85" s="1223" t="n"/>
-      <c r="J85" s="1224" t="n"/>
-      <c r="K85" s="1303" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
-      <c r="L85" s="1304" t="n"/>
-      <c r="M85" s="1223" t="n"/>
-      <c r="N85" s="1223" t="n"/>
-      <c r="O85" s="1223" t="n"/>
-      <c r="P85" s="1224" t="n"/>
+    <row r="85" ht="15.75" customFormat="1" customHeight="1" s="1221">
+      <c r="A85" s="1215" t="inlineStr">
+        <is>
+          <t>Dry yeast</t>
+        </is>
+      </c>
+      <c r="B85" s="1114" t="n"/>
+      <c r="C85" s="1114" t="n"/>
+      <c r="D85" s="1114" t="n"/>
+      <c r="E85" s="1114" t="n"/>
+      <c r="F85" s="1114" t="n"/>
+      <c r="G85" s="1114" t="n"/>
+      <c r="H85" s="1114" t="n"/>
+      <c r="I85" s="1114" t="n"/>
+      <c r="J85" s="1114" t="n"/>
+      <c r="K85" s="1114" t="n"/>
+      <c r="L85" s="1114" t="n"/>
+      <c r="M85" s="1114" t="n"/>
+      <c r="N85" s="1114" t="n"/>
+      <c r="O85" s="1114" t="n"/>
+      <c r="P85" s="1115" t="n"/>
       <c r="Q85" s="1138" t="n"/>
       <c r="R85" s="1139" t="n"/>
       <c r="S85" s="1139" t="n"/>
@@ -12813,53 +12791,67 @@
       <c r="U85" s="1188" t="n"/>
     </row>
     <row r="86" ht="15" customFormat="1" customHeight="1" s="1221">
-      <c r="A86" s="1236" t="n"/>
-      <c r="B86" s="1198" t="n"/>
-      <c r="C86" s="1198" t="n"/>
-      <c r="D86" s="1198" t="n"/>
-      <c r="E86" s="1198" t="n"/>
-      <c r="F86" s="1199" t="n"/>
-      <c r="G86" s="1305" t="n"/>
-      <c r="H86" s="1198" t="n"/>
-      <c r="I86" s="1198" t="n"/>
-      <c r="J86" s="1199" t="n"/>
-      <c r="K86" s="1305" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
-      <c r="L86" s="1306" t="n"/>
-      <c r="M86" s="1198" t="n"/>
-      <c r="N86" s="1198" t="n"/>
-      <c r="O86" s="1198" t="n"/>
-      <c r="P86" s="1199" t="n"/>
+      <c r="A86" s="1296" t="inlineStr">
+        <is>
+          <t>Soort</t>
+        </is>
+      </c>
+      <c r="B86" s="1114" t="n"/>
+      <c r="C86" s="1114" t="n"/>
+      <c r="D86" s="1114" t="n"/>
+      <c r="E86" s="1114" t="n"/>
+      <c r="F86" s="1297" t="inlineStr">
+        <is>
+          <t>Brews/1st day</t>
+        </is>
+      </c>
+      <c r="G86" s="1298" t="inlineStr">
+        <is>
+          <t>Hoeveelheid per batch</t>
+        </is>
+      </c>
+      <c r="H86" s="1114" t="n"/>
+      <c r="I86" s="1114" t="n"/>
+      <c r="J86" s="1114" t="n"/>
+      <c r="K86" s="1115" t="n"/>
+      <c r="L86" s="1299" t="inlineStr">
+        <is>
+          <t>Lotnummer</t>
+        </is>
+      </c>
+      <c r="M86" s="1080" t="n"/>
+      <c r="N86" s="1080" t="n"/>
+      <c r="O86" s="1080" t="n"/>
+      <c r="P86" s="1081" t="n"/>
       <c r="Q86" s="1138" t="n"/>
       <c r="R86" s="1139" t="n"/>
       <c r="S86" s="1139" t="n"/>
       <c r="T86" s="1139" t="n"/>
       <c r="U86" s="1188" t="n"/>
     </row>
-    <row r="87" ht="18.75" customFormat="1" customHeight="1" s="1221">
-      <c r="A87" s="1307" t="inlineStr">
-        <is>
-          <t>Additions Cellar</t>
-        </is>
-      </c>
-      <c r="B87" s="1114" t="n"/>
-      <c r="C87" s="1114" t="n"/>
-      <c r="D87" s="1114" t="n"/>
-      <c r="E87" s="1114" t="n"/>
-      <c r="F87" s="1114" t="n"/>
-      <c r="G87" s="1114" t="n"/>
-      <c r="H87" s="1114" t="n"/>
-      <c r="I87" s="1114" t="n"/>
-      <c r="J87" s="1114" t="n"/>
-      <c r="K87" s="1114" t="n"/>
-      <c r="L87" s="1114" t="n"/>
-      <c r="M87" s="1114" t="n"/>
-      <c r="N87" s="1114" t="n"/>
-      <c r="O87" s="1114" t="n"/>
-      <c r="P87" s="1115" t="n"/>
+    <row r="87" ht="15" customFormat="1" customHeight="1" s="1221">
+      <c r="A87" s="1300" t="n"/>
+      <c r="B87" s="1223" t="n"/>
+      <c r="C87" s="1223" t="n"/>
+      <c r="D87" s="1223" t="n"/>
+      <c r="E87" s="1223" t="n"/>
+      <c r="F87" s="1301" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" s="1302" t="n"/>
+      <c r="H87" s="1223" t="n"/>
+      <c r="I87" s="1223" t="n"/>
+      <c r="J87" s="1224" t="n"/>
+      <c r="K87" s="1303" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="L87" s="1304" t="n"/>
+      <c r="M87" s="1223" t="n"/>
+      <c r="N87" s="1223" t="n"/>
+      <c r="O87" s="1223" t="n"/>
+      <c r="P87" s="1224" t="n"/>
       <c r="Q87" s="1138" t="n"/>
       <c r="R87" s="1139" t="n"/>
       <c r="S87" s="1139" t="n"/>
@@ -12867,61 +12859,53 @@
       <c r="U87" s="1188" t="n"/>
     </row>
     <row r="88" ht="15" customFormat="1" customHeight="1" s="1221">
-      <c r="A88" s="1285" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B88" s="1114" t="n"/>
-      <c r="C88" s="1114" t="n"/>
-      <c r="D88" s="1115" t="n"/>
-      <c r="E88" s="1286" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="F88" s="1114" t="n"/>
-      <c r="G88" s="1114" t="n"/>
-      <c r="H88" s="1114" t="n"/>
-      <c r="I88" s="1287" t="inlineStr">
-        <is>
-          <t>When</t>
-        </is>
-      </c>
-      <c r="J88" s="1114" t="n"/>
-      <c r="K88" s="1115" t="n"/>
-      <c r="L88" s="1288" t="inlineStr">
-        <is>
-          <t>Lotnummer</t>
-        </is>
-      </c>
-      <c r="M88" s="1080" t="n"/>
-      <c r="N88" s="1080" t="n"/>
-      <c r="O88" s="1080" t="n"/>
-      <c r="P88" s="1081" t="n"/>
+      <c r="A88" s="1236" t="n"/>
+      <c r="B88" s="1198" t="n"/>
+      <c r="C88" s="1198" t="n"/>
+      <c r="D88" s="1198" t="n"/>
+      <c r="E88" s="1198" t="n"/>
+      <c r="F88" s="1199" t="n"/>
+      <c r="G88" s="1305" t="n"/>
+      <c r="H88" s="1198" t="n"/>
+      <c r="I88" s="1198" t="n"/>
+      <c r="J88" s="1199" t="n"/>
+      <c r="K88" s="1305" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="L88" s="1306" t="n"/>
+      <c r="M88" s="1198" t="n"/>
+      <c r="N88" s="1198" t="n"/>
+      <c r="O88" s="1198" t="n"/>
+      <c r="P88" s="1199" t="n"/>
       <c r="Q88" s="1138" t="n"/>
       <c r="R88" s="1139" t="n"/>
       <c r="S88" s="1139" t="n"/>
       <c r="T88" s="1139" t="n"/>
       <c r="U88" s="1188" t="n"/>
     </row>
-    <row r="89" ht="15" customFormat="1" customHeight="1" s="1221">
-      <c r="A89" s="1289" t="n"/>
-      <c r="B89" s="1177" t="n"/>
-      <c r="C89" s="1177" t="n"/>
-      <c r="D89" s="1178" t="n"/>
-      <c r="E89" s="1308" t="n"/>
-      <c r="F89" s="1177" t="n"/>
-      <c r="G89" s="1177" t="n"/>
-      <c r="H89" s="1177" t="n"/>
-      <c r="I89" s="1291" t="n"/>
-      <c r="J89" s="1223" t="n"/>
-      <c r="K89" s="1224" t="n"/>
-      <c r="L89" s="1309" t="n"/>
-      <c r="M89" s="1223" t="n"/>
-      <c r="N89" s="1223" t="n"/>
-      <c r="O89" s="1223" t="n"/>
-      <c r="P89" s="1224" t="n"/>
+    <row r="89" ht="18.75" customFormat="1" customHeight="1" s="1221">
+      <c r="A89" s="1307" t="inlineStr">
+        <is>
+          <t>Additions Cellar</t>
+        </is>
+      </c>
+      <c r="B89" s="1114" t="n"/>
+      <c r="C89" s="1114" t="n"/>
+      <c r="D89" s="1114" t="n"/>
+      <c r="E89" s="1114" t="n"/>
+      <c r="F89" s="1114" t="n"/>
+      <c r="G89" s="1114" t="n"/>
+      <c r="H89" s="1114" t="n"/>
+      <c r="I89" s="1114" t="n"/>
+      <c r="J89" s="1114" t="n"/>
+      <c r="K89" s="1114" t="n"/>
+      <c r="L89" s="1114" t="n"/>
+      <c r="M89" s="1114" t="n"/>
+      <c r="N89" s="1114" t="n"/>
+      <c r="O89" s="1114" t="n"/>
+      <c r="P89" s="1115" t="n"/>
       <c r="Q89" s="1138" t="n"/>
       <c r="R89" s="1139" t="n"/>
       <c r="S89" s="1139" t="n"/>
@@ -12929,29 +12913,45 @@
       <c r="U89" s="1188" t="n"/>
     </row>
     <row r="90" ht="15" customFormat="1" customHeight="1" s="1221">
-      <c r="A90" s="1289" t="n"/>
-      <c r="B90" s="1177" t="n"/>
-      <c r="C90" s="1177" t="n"/>
-      <c r="D90" s="1178" t="n"/>
-      <c r="E90" s="1308" t="n"/>
-      <c r="F90" s="1177" t="n"/>
-      <c r="G90" s="1177" t="n"/>
-      <c r="H90" s="1177" t="n"/>
-      <c r="I90" s="1289" t="n"/>
-      <c r="J90" s="1177" t="n"/>
-      <c r="K90" s="1178" t="n"/>
-      <c r="L90" s="1292" t="n"/>
-      <c r="M90" s="1177" t="n"/>
-      <c r="N90" s="1177" t="n"/>
-      <c r="O90" s="1177" t="n"/>
-      <c r="P90" s="1178" t="n"/>
+      <c r="A90" s="1285" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B90" s="1114" t="n"/>
+      <c r="C90" s="1114" t="n"/>
+      <c r="D90" s="1115" t="n"/>
+      <c r="E90" s="1286" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="F90" s="1114" t="n"/>
+      <c r="G90" s="1114" t="n"/>
+      <c r="H90" s="1114" t="n"/>
+      <c r="I90" s="1287" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+      <c r="J90" s="1114" t="n"/>
+      <c r="K90" s="1115" t="n"/>
+      <c r="L90" s="1288" t="inlineStr">
+        <is>
+          <t>Lotnummer</t>
+        </is>
+      </c>
+      <c r="M90" s="1080" t="n"/>
+      <c r="N90" s="1080" t="n"/>
+      <c r="O90" s="1080" t="n"/>
+      <c r="P90" s="1081" t="n"/>
       <c r="Q90" s="1138" t="n"/>
       <c r="R90" s="1139" t="n"/>
       <c r="S90" s="1139" t="n"/>
       <c r="T90" s="1139" t="n"/>
       <c r="U90" s="1188" t="n"/>
     </row>
-    <row r="91" ht="15" customFormat="1" customHeight="1" s="1310">
+    <row r="91" ht="15" customFormat="1" customHeight="1" s="1221">
       <c r="A91" s="1289" t="n"/>
       <c r="B91" s="1177" t="n"/>
       <c r="C91" s="1177" t="n"/>
@@ -12960,21 +12960,21 @@
       <c r="F91" s="1177" t="n"/>
       <c r="G91" s="1177" t="n"/>
       <c r="H91" s="1177" t="n"/>
-      <c r="I91" s="1289" t="n"/>
-      <c r="J91" s="1177" t="n"/>
-      <c r="K91" s="1178" t="n"/>
-      <c r="L91" s="1292" t="n"/>
-      <c r="M91" s="1177" t="n"/>
-      <c r="N91" s="1177" t="n"/>
-      <c r="O91" s="1177" t="n"/>
-      <c r="P91" s="1178" t="n"/>
+      <c r="I91" s="1291" t="n"/>
+      <c r="J91" s="1223" t="n"/>
+      <c r="K91" s="1224" t="n"/>
+      <c r="L91" s="1309" t="n"/>
+      <c r="M91" s="1223" t="n"/>
+      <c r="N91" s="1223" t="n"/>
+      <c r="O91" s="1223" t="n"/>
+      <c r="P91" s="1224" t="n"/>
       <c r="Q91" s="1138" t="n"/>
       <c r="R91" s="1139" t="n"/>
       <c r="S91" s="1139" t="n"/>
       <c r="T91" s="1139" t="n"/>
       <c r="U91" s="1188" t="n"/>
     </row>
-    <row r="92" ht="15" customFormat="1" customHeight="1" s="1310">
+    <row r="92" ht="15" customFormat="1" customHeight="1" s="1221">
       <c r="A92" s="1289" t="n"/>
       <c r="B92" s="1177" t="n"/>
       <c r="C92" s="1177" t="n"/>
@@ -13006,115 +13006,87 @@
       <c r="F93" s="1177" t="n"/>
       <c r="G93" s="1177" t="n"/>
       <c r="H93" s="1177" t="n"/>
-      <c r="I93" s="1311" t="n"/>
-      <c r="J93" s="1198" t="n"/>
-      <c r="K93" s="1199" t="n"/>
-      <c r="L93" s="1312" t="n"/>
-      <c r="M93" s="1198" t="n"/>
-      <c r="N93" s="1198" t="n"/>
-      <c r="O93" s="1198" t="n"/>
-      <c r="P93" s="1199" t="n"/>
+      <c r="I93" s="1289" t="n"/>
+      <c r="J93" s="1177" t="n"/>
+      <c r="K93" s="1178" t="n"/>
+      <c r="L93" s="1292" t="n"/>
+      <c r="M93" s="1177" t="n"/>
+      <c r="N93" s="1177" t="n"/>
+      <c r="O93" s="1177" t="n"/>
+      <c r="P93" s="1178" t="n"/>
       <c r="Q93" s="1138" t="n"/>
       <c r="R93" s="1139" t="n"/>
       <c r="S93" s="1139" t="n"/>
       <c r="T93" s="1139" t="n"/>
       <c r="U93" s="1188" t="n"/>
     </row>
-    <row r="94" ht="18.75" customFormat="1" customHeight="1" s="1313">
-      <c r="A94" s="1314" t="inlineStr">
+    <row r="94" ht="15" customFormat="1" customHeight="1" s="1310">
+      <c r="A94" s="1289" t="n"/>
+      <c r="B94" s="1177" t="n"/>
+      <c r="C94" s="1177" t="n"/>
+      <c r="D94" s="1178" t="n"/>
+      <c r="E94" s="1308" t="n"/>
+      <c r="F94" s="1177" t="n"/>
+      <c r="G94" s="1177" t="n"/>
+      <c r="H94" s="1177" t="n"/>
+      <c r="I94" s="1289" t="n"/>
+      <c r="J94" s="1177" t="n"/>
+      <c r="K94" s="1178" t="n"/>
+      <c r="L94" s="1292" t="n"/>
+      <c r="M94" s="1177" t="n"/>
+      <c r="N94" s="1177" t="n"/>
+      <c r="O94" s="1177" t="n"/>
+      <c r="P94" s="1178" t="n"/>
+      <c r="Q94" s="1138" t="n"/>
+      <c r="R94" s="1139" t="n"/>
+      <c r="S94" s="1139" t="n"/>
+      <c r="T94" s="1139" t="n"/>
+      <c r="U94" s="1188" t="n"/>
+    </row>
+    <row r="95" ht="15" customFormat="1" customHeight="1" s="1310">
+      <c r="A95" s="1289" t="n"/>
+      <c r="B95" s="1177" t="n"/>
+      <c r="C95" s="1177" t="n"/>
+      <c r="D95" s="1178" t="n"/>
+      <c r="E95" s="1308" t="n"/>
+      <c r="F95" s="1177" t="n"/>
+      <c r="G95" s="1177" t="n"/>
+      <c r="H95" s="1177" t="n"/>
+      <c r="I95" s="1311" t="n"/>
+      <c r="J95" s="1198" t="n"/>
+      <c r="K95" s="1199" t="n"/>
+      <c r="L95" s="1312" t="n"/>
+      <c r="M95" s="1198" t="n"/>
+      <c r="N95" s="1198" t="n"/>
+      <c r="O95" s="1198" t="n"/>
+      <c r="P95" s="1199" t="n"/>
+      <c r="Q95" s="1138" t="n"/>
+      <c r="R95" s="1139" t="n"/>
+      <c r="S95" s="1139" t="n"/>
+      <c r="T95" s="1139" t="n"/>
+      <c r="U95" s="1188" t="n"/>
+    </row>
+    <row r="96" ht="18.75" customFormat="1" customHeight="1" s="1313">
+      <c r="A96" s="1314" t="inlineStr">
         <is>
           <t>Target Water Profile(values in PPM)</t>
         </is>
       </c>
-      <c r="B94" s="1315" t="n"/>
-      <c r="C94" s="1315" t="n"/>
-      <c r="D94" s="1315" t="n"/>
-      <c r="E94" s="1315" t="n"/>
-      <c r="F94" s="1315" t="n"/>
-      <c r="G94" s="1315" t="n"/>
-      <c r="H94" s="1315" t="n"/>
-      <c r="I94" s="1315" t="n"/>
-      <c r="J94" s="1315" t="n"/>
-      <c r="K94" s="1315" t="n"/>
-      <c r="L94" s="1315" t="n"/>
-      <c r="M94" s="1315" t="n"/>
-      <c r="N94" s="1315" t="n"/>
-      <c r="O94" s="1315" t="n"/>
-      <c r="P94" s="1316" t="n"/>
-      <c r="Q94" s="1317" t="n"/>
-      <c r="R94" s="1318" t="n"/>
-      <c r="S94" s="1318" t="n"/>
-      <c r="T94" s="1318" t="n"/>
-      <c r="U94" s="1319" t="n"/>
-    </row>
-    <row r="95" ht="12.75" customFormat="1" customHeight="1" s="1313">
-      <c r="A95" s="1320" t="inlineStr">
-        <is>
-          <t>Ca</t>
-        </is>
-      </c>
-      <c r="B95" s="1321" t="n"/>
-      <c r="C95" s="1321" t="inlineStr">
-        <is>
-          <t>Mg</t>
-        </is>
-      </c>
-      <c r="D95" s="1321" t="n"/>
-      <c r="E95" s="1321" t="inlineStr">
-        <is>
-          <t>Na</t>
-        </is>
-      </c>
-      <c r="F95" s="1321" t="n"/>
-      <c r="G95" s="1321" t="inlineStr">
-        <is>
-          <t>Cl</t>
-        </is>
-      </c>
-      <c r="H95" s="1321" t="n"/>
-      <c r="I95" s="1321" t="n"/>
-      <c r="J95" s="1321" t="inlineStr">
-        <is>
-          <t>SO4</t>
-        </is>
-      </c>
-      <c r="K95" s="1321" t="n"/>
-      <c r="L95" s="1321" t="n"/>
-      <c r="M95" s="1321" t="inlineStr">
-        <is>
-          <t>Ratio Cl:SO4</t>
-        </is>
-      </c>
-      <c r="N95" s="1321" t="n"/>
-      <c r="O95" s="1321" t="n"/>
-      <c r="P95" s="1322" t="inlineStr">
-        <is>
-          <t>Alkalinity</t>
-        </is>
-      </c>
-      <c r="Q95" s="1317" t="n"/>
-      <c r="R95" s="1318" t="n"/>
-      <c r="S95" s="1318" t="n"/>
-      <c r="T95" s="1318" t="n"/>
-      <c r="U95" s="1319" t="n"/>
-    </row>
-    <row r="96" ht="5.25" customFormat="1" customHeight="1" s="1313">
-      <c r="A96" s="1323" t="n"/>
-      <c r="B96" s="1324" t="n"/>
-      <c r="C96" s="1324" t="n"/>
-      <c r="D96" s="1324" t="n"/>
-      <c r="E96" s="1324" t="n"/>
-      <c r="F96" s="1324" t="n"/>
-      <c r="G96" s="1324" t="n"/>
-      <c r="H96" s="1324" t="n"/>
-      <c r="I96" s="1324" t="n"/>
-      <c r="J96" s="1324" t="n"/>
-      <c r="K96" s="1324" t="n"/>
-      <c r="L96" s="1324" t="n"/>
-      <c r="M96" s="1324" t="n"/>
-      <c r="N96" s="1324" t="n"/>
-      <c r="O96" s="1324" t="n"/>
-      <c r="P96" s="1325" t="n"/>
+      <c r="B96" s="1315" t="n"/>
+      <c r="C96" s="1315" t="n"/>
+      <c r="D96" s="1315" t="n"/>
+      <c r="E96" s="1315" t="n"/>
+      <c r="F96" s="1315" t="n"/>
+      <c r="G96" s="1315" t="n"/>
+      <c r="H96" s="1315" t="n"/>
+      <c r="I96" s="1315" t="n"/>
+      <c r="J96" s="1315" t="n"/>
+      <c r="K96" s="1315" t="n"/>
+      <c r="L96" s="1315" t="n"/>
+      <c r="M96" s="1315" t="n"/>
+      <c r="N96" s="1315" t="n"/>
+      <c r="O96" s="1315" t="n"/>
+      <c r="P96" s="1316" t="n"/>
       <c r="Q96" s="1317" t="n"/>
       <c r="R96" s="1318" t="n"/>
       <c r="S96" s="1318" t="n"/>
@@ -13122,157 +13094,185 @@
       <c r="U96" s="1319" t="n"/>
     </row>
     <row r="97" ht="12.75" customFormat="1" customHeight="1" s="1313">
-      <c r="A97" s="1326" t="n"/>
-      <c r="B97" s="1326" t="n"/>
-      <c r="C97" s="1326" t="n"/>
-      <c r="D97" s="1326" t="n"/>
-      <c r="E97" s="1326" t="n"/>
-      <c r="F97" s="1326" t="n"/>
-      <c r="G97" s="1326" t="n"/>
-      <c r="H97" s="1326" t="n"/>
-      <c r="I97" s="1326" t="n"/>
-      <c r="J97" s="1326" t="n"/>
-      <c r="K97" s="1326" t="n"/>
-      <c r="L97" s="1326" t="n"/>
-      <c r="M97" s="1327" t="n"/>
-      <c r="N97" s="1326" t="n"/>
-      <c r="O97" s="1326" t="n"/>
-      <c r="P97" s="1328" t="n"/>
+      <c r="A97" s="1320" t="inlineStr">
+        <is>
+          <t>Ca</t>
+        </is>
+      </c>
+      <c r="B97" s="1321" t="n"/>
+      <c r="C97" s="1321" t="inlineStr">
+        <is>
+          <t>Mg</t>
+        </is>
+      </c>
+      <c r="D97" s="1321" t="n"/>
+      <c r="E97" s="1321" t="inlineStr">
+        <is>
+          <t>Na</t>
+        </is>
+      </c>
+      <c r="F97" s="1321" t="n"/>
+      <c r="G97" s="1321" t="inlineStr">
+        <is>
+          <t>Cl</t>
+        </is>
+      </c>
+      <c r="H97" s="1321" t="n"/>
+      <c r="I97" s="1321" t="n"/>
+      <c r="J97" s="1321" t="inlineStr">
+        <is>
+          <t>SO4</t>
+        </is>
+      </c>
+      <c r="K97" s="1321" t="n"/>
+      <c r="L97" s="1321" t="n"/>
+      <c r="M97" s="1321" t="inlineStr">
+        <is>
+          <t>Ratio Cl:SO4</t>
+        </is>
+      </c>
+      <c r="N97" s="1321" t="n"/>
+      <c r="O97" s="1321" t="n"/>
+      <c r="P97" s="1322" t="inlineStr">
+        <is>
+          <t>Alkalinity</t>
+        </is>
+      </c>
       <c r="Q97" s="1317" t="n"/>
       <c r="R97" s="1318" t="n"/>
       <c r="S97" s="1318" t="n"/>
       <c r="T97" s="1318" t="n"/>
       <c r="U97" s="1319" t="n"/>
     </row>
-    <row r="98" ht="6" customFormat="1" customHeight="1" s="1313">
-      <c r="A98" s="1329" t="n"/>
-      <c r="B98" s="1093" t="n"/>
-      <c r="C98" s="1093" t="n"/>
-      <c r="D98" s="1093" t="n"/>
-      <c r="E98" s="1093" t="n"/>
-      <c r="F98" s="1093" t="n"/>
-      <c r="G98" s="1093" t="n"/>
-      <c r="H98" s="1093" t="n"/>
-      <c r="I98" s="1093" t="n"/>
-      <c r="J98" s="1093" t="n"/>
-      <c r="K98" s="1093" t="n"/>
-      <c r="L98" s="1093" t="n"/>
-      <c r="M98" s="1093" t="n"/>
-      <c r="N98" s="1093" t="n"/>
-      <c r="O98" s="1093" t="n"/>
-      <c r="P98" s="1094" t="n"/>
+    <row r="98" ht="5.25" customFormat="1" customHeight="1" s="1313">
+      <c r="A98" s="1323" t="n"/>
+      <c r="B98" s="1324" t="n"/>
+      <c r="C98" s="1324" t="n"/>
+      <c r="D98" s="1324" t="n"/>
+      <c r="E98" s="1324" t="n"/>
+      <c r="F98" s="1324" t="n"/>
+      <c r="G98" s="1324" t="n"/>
+      <c r="H98" s="1324" t="n"/>
+      <c r="I98" s="1324" t="n"/>
+      <c r="J98" s="1324" t="n"/>
+      <c r="K98" s="1324" t="n"/>
+      <c r="L98" s="1324" t="n"/>
+      <c r="M98" s="1324" t="n"/>
+      <c r="N98" s="1324" t="n"/>
+      <c r="O98" s="1324" t="n"/>
+      <c r="P98" s="1325" t="n"/>
       <c r="Q98" s="1317" t="n"/>
       <c r="R98" s="1318" t="n"/>
       <c r="S98" s="1318" t="n"/>
       <c r="T98" s="1318" t="n"/>
       <c r="U98" s="1319" t="n"/>
     </row>
-    <row r="99" ht="18.75" customFormat="1" customHeight="1" s="1310">
-      <c r="A99" s="1330" t="inlineStr">
+    <row r="99" ht="12.75" customFormat="1" customHeight="1" s="1313">
+      <c r="A99" s="1326" t="n"/>
+      <c r="B99" s="1326" t="n"/>
+      <c r="C99" s="1326" t="n"/>
+      <c r="D99" s="1326" t="n"/>
+      <c r="E99" s="1326" t="n"/>
+      <c r="F99" s="1326" t="n"/>
+      <c r="G99" s="1326" t="n"/>
+      <c r="H99" s="1326" t="n"/>
+      <c r="I99" s="1326" t="n"/>
+      <c r="J99" s="1326" t="n"/>
+      <c r="K99" s="1326" t="n"/>
+      <c r="L99" s="1326" t="n"/>
+      <c r="M99" s="1327" t="n"/>
+      <c r="N99" s="1326" t="n"/>
+      <c r="O99" s="1326" t="n"/>
+      <c r="P99" s="1328" t="n"/>
+      <c r="Q99" s="1317" t="n"/>
+      <c r="R99" s="1318" t="n"/>
+      <c r="S99" s="1318" t="n"/>
+      <c r="T99" s="1318" t="n"/>
+      <c r="U99" s="1319" t="n"/>
+    </row>
+    <row r="100" ht="6" customFormat="1" customHeight="1" s="1313">
+      <c r="A100" s="1329" t="n"/>
+      <c r="B100" s="1093" t="n"/>
+      <c r="C100" s="1093" t="n"/>
+      <c r="D100" s="1093" t="n"/>
+      <c r="E100" s="1093" t="n"/>
+      <c r="F100" s="1093" t="n"/>
+      <c r="G100" s="1093" t="n"/>
+      <c r="H100" s="1093" t="n"/>
+      <c r="I100" s="1093" t="n"/>
+      <c r="J100" s="1093" t="n"/>
+      <c r="K100" s="1093" t="n"/>
+      <c r="L100" s="1093" t="n"/>
+      <c r="M100" s="1093" t="n"/>
+      <c r="N100" s="1093" t="n"/>
+      <c r="O100" s="1093" t="n"/>
+      <c r="P100" s="1094" t="n"/>
+      <c r="Q100" s="1317" t="n"/>
+      <c r="R100" s="1318" t="n"/>
+      <c r="S100" s="1318" t="n"/>
+      <c r="T100" s="1318" t="n"/>
+      <c r="U100" s="1319" t="n"/>
+    </row>
+    <row r="101" ht="18.75" customFormat="1" customHeight="1" s="1310">
+      <c r="A101" s="1330" t="inlineStr">
         <is>
           <t>Revisie nummer</t>
         </is>
       </c>
-      <c r="B99" s="1114" t="n"/>
-      <c r="C99" s="1114" t="n"/>
-      <c r="D99" s="1114" t="n"/>
-      <c r="E99" s="1114" t="n"/>
-      <c r="F99" s="1114" t="n"/>
-      <c r="G99" s="1114" t="n"/>
-      <c r="H99" s="1114" t="n"/>
-      <c r="I99" s="1114" t="n"/>
-      <c r="J99" s="1114" t="n"/>
-      <c r="K99" s="1114" t="n"/>
-      <c r="L99" s="1114" t="n"/>
-      <c r="M99" s="1114" t="n"/>
-      <c r="N99" s="1114" t="n"/>
-      <c r="O99" s="1114" t="n"/>
-      <c r="P99" s="1115" t="n"/>
-      <c r="Q99" s="1138" t="n"/>
-      <c r="R99" s="1139" t="n"/>
-      <c r="S99" s="1139" t="n"/>
-      <c r="T99" s="1139" t="n"/>
-      <c r="U99" s="1187" t="n"/>
-    </row>
-    <row r="100" ht="15" customFormat="1" customHeight="1" s="1331">
-      <c r="A100" s="1298" t="inlineStr">
-        <is>
-          <t>Revisie nummer</t>
-        </is>
-      </c>
-      <c r="B100" s="1114" t="n"/>
-      <c r="C100" s="1115" t="n"/>
-      <c r="D100" s="1332" t="inlineStr">
-        <is>
-          <t>Wijziging</t>
-        </is>
-      </c>
-      <c r="E100" s="1333" t="n"/>
-      <c r="F100" s="1333" t="n"/>
-      <c r="G100" s="1333" t="n"/>
-      <c r="H100" s="1333" t="n"/>
-      <c r="I100" s="1333" t="n"/>
-      <c r="J100" s="1333" t="n"/>
-      <c r="K100" s="1333" t="n"/>
-      <c r="L100" s="1333" t="n"/>
-      <c r="M100" s="1333" t="n"/>
-      <c r="N100" s="1296" t="inlineStr">
-        <is>
-          <t>Datum</t>
-        </is>
-      </c>
-      <c r="O100" s="1114" t="n"/>
-      <c r="P100" s="1334" t="inlineStr">
-        <is>
-          <t>Door</t>
-        </is>
-      </c>
-      <c r="Q100" s="1138" t="n"/>
-      <c r="R100" s="1139" t="n"/>
-      <c r="S100" s="1139" t="n"/>
-      <c r="T100" s="1139" t="n"/>
-      <c r="U100" s="1157" t="n"/>
-    </row>
-    <row r="101" ht="15" customFormat="1" customHeight="1" s="1073">
-      <c r="A101" s="1335" t="n"/>
-      <c r="B101" s="1223" t="n"/>
-      <c r="C101" s="1224" t="n"/>
-      <c r="D101" s="1233" t="n"/>
-      <c r="E101" s="1177" t="n"/>
-      <c r="F101" s="1177" t="n"/>
-      <c r="G101" s="1177" t="n"/>
-      <c r="H101" s="1177" t="n"/>
-      <c r="I101" s="1177" t="n"/>
-      <c r="J101" s="1177" t="n"/>
-      <c r="K101" s="1177" t="n"/>
-      <c r="L101" s="1177" t="n"/>
-      <c r="M101" s="1178" t="n"/>
-      <c r="N101" s="1336" t="n"/>
-      <c r="O101" s="1224" t="n"/>
-      <c r="P101" s="1303" t="n"/>
+      <c r="B101" s="1114" t="n"/>
+      <c r="C101" s="1114" t="n"/>
+      <c r="D101" s="1114" t="n"/>
+      <c r="E101" s="1114" t="n"/>
+      <c r="F101" s="1114" t="n"/>
+      <c r="G101" s="1114" t="n"/>
+      <c r="H101" s="1114" t="n"/>
+      <c r="I101" s="1114" t="n"/>
+      <c r="J101" s="1114" t="n"/>
+      <c r="K101" s="1114" t="n"/>
+      <c r="L101" s="1114" t="n"/>
+      <c r="M101" s="1114" t="n"/>
+      <c r="N101" s="1114" t="n"/>
+      <c r="O101" s="1114" t="n"/>
+      <c r="P101" s="1115" t="n"/>
       <c r="Q101" s="1138" t="n"/>
       <c r="R101" s="1139" t="n"/>
       <c r="S101" s="1139" t="n"/>
       <c r="T101" s="1139" t="n"/>
-      <c r="U101" s="1157" t="n"/>
-    </row>
-    <row r="102" ht="15" customFormat="1" customHeight="1" s="1073">
-      <c r="A102" s="1337" t="n"/>
-      <c r="B102" s="1177" t="n"/>
-      <c r="C102" s="1178" t="n"/>
-      <c r="D102" s="1233" t="n"/>
-      <c r="E102" s="1177" t="n"/>
-      <c r="F102" s="1177" t="n"/>
-      <c r="G102" s="1177" t="n"/>
-      <c r="H102" s="1177" t="n"/>
-      <c r="I102" s="1177" t="n"/>
-      <c r="J102" s="1177" t="n"/>
-      <c r="K102" s="1177" t="n"/>
-      <c r="L102" s="1177" t="n"/>
-      <c r="M102" s="1178" t="n"/>
-      <c r="N102" s="1338" t="n"/>
-      <c r="O102" s="1178" t="n"/>
-      <c r="P102" s="1337" t="n"/>
+      <c r="U101" s="1187" t="n"/>
+    </row>
+    <row r="102" ht="15" customFormat="1" customHeight="1" s="1331">
+      <c r="A102" s="1298" t="inlineStr">
+        <is>
+          <t>Revisie nummer</t>
+        </is>
+      </c>
+      <c r="B102" s="1114" t="n"/>
+      <c r="C102" s="1115" t="n"/>
+      <c r="D102" s="1332" t="inlineStr">
+        <is>
+          <t>Wijziging</t>
+        </is>
+      </c>
+      <c r="E102" s="1333" t="n"/>
+      <c r="F102" s="1333" t="n"/>
+      <c r="G102" s="1333" t="n"/>
+      <c r="H102" s="1333" t="n"/>
+      <c r="I102" s="1333" t="n"/>
+      <c r="J102" s="1333" t="n"/>
+      <c r="K102" s="1333" t="n"/>
+      <c r="L102" s="1333" t="n"/>
+      <c r="M102" s="1333" t="n"/>
+      <c r="N102" s="1296" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="O102" s="1114" t="n"/>
+      <c r="P102" s="1334" t="inlineStr">
+        <is>
+          <t>Door</t>
+        </is>
+      </c>
       <c r="Q102" s="1138" t="n"/>
       <c r="R102" s="1139" t="n"/>
       <c r="S102" s="1139" t="n"/>
@@ -13280,9 +13280,9 @@
       <c r="U102" s="1157" t="n"/>
     </row>
     <row r="103" ht="15" customFormat="1" customHeight="1" s="1073">
-      <c r="A103" s="1337" t="n"/>
-      <c r="B103" s="1177" t="n"/>
-      <c r="C103" s="1178" t="n"/>
+      <c r="A103" s="1335" t="n"/>
+      <c r="B103" s="1223" t="n"/>
+      <c r="C103" s="1224" t="n"/>
       <c r="D103" s="1233" t="n"/>
       <c r="E103" s="1177" t="n"/>
       <c r="F103" s="1177" t="n"/>
@@ -13293,9 +13293,9 @@
       <c r="K103" s="1177" t="n"/>
       <c r="L103" s="1177" t="n"/>
       <c r="M103" s="1178" t="n"/>
-      <c r="N103" s="1338" t="n"/>
-      <c r="O103" s="1178" t="n"/>
-      <c r="P103" s="1337" t="n"/>
+      <c r="N103" s="1336" t="n"/>
+      <c r="O103" s="1224" t="n"/>
+      <c r="P103" s="1303" t="n"/>
       <c r="Q103" s="1138" t="n"/>
       <c r="R103" s="1139" t="n"/>
       <c r="S103" s="1139" t="n"/>
@@ -13326,146 +13326,192 @@
       <c r="U104" s="1157" t="n"/>
     </row>
     <row r="105" ht="15" customFormat="1" customHeight="1" s="1073">
-      <c r="A105" s="1305" t="n"/>
-      <c r="B105" s="1198" t="n"/>
-      <c r="C105" s="1199" t="n"/>
-      <c r="D105" s="1305" t="n"/>
-      <c r="E105" s="1198" t="n"/>
-      <c r="F105" s="1198" t="n"/>
-      <c r="G105" s="1198" t="n"/>
-      <c r="H105" s="1198" t="n"/>
-      <c r="I105" s="1198" t="n"/>
-      <c r="J105" s="1198" t="n"/>
-      <c r="K105" s="1198" t="n"/>
-      <c r="L105" s="1198" t="n"/>
-      <c r="M105" s="1198" t="n"/>
-      <c r="N105" s="1198" t="n"/>
-      <c r="O105" s="1198" t="n"/>
-      <c r="P105" s="1199" t="n"/>
+      <c r="A105" s="1337" t="n"/>
+      <c r="B105" s="1177" t="n"/>
+      <c r="C105" s="1178" t="n"/>
+      <c r="D105" s="1233" t="n"/>
+      <c r="E105" s="1177" t="n"/>
+      <c r="F105" s="1177" t="n"/>
+      <c r="G105" s="1177" t="n"/>
+      <c r="H105" s="1177" t="n"/>
+      <c r="I105" s="1177" t="n"/>
+      <c r="J105" s="1177" t="n"/>
+      <c r="K105" s="1177" t="n"/>
+      <c r="L105" s="1177" t="n"/>
+      <c r="M105" s="1178" t="n"/>
+      <c r="N105" s="1338" t="n"/>
+      <c r="O105" s="1178" t="n"/>
+      <c r="P105" s="1337" t="n"/>
       <c r="Q105" s="1138" t="n"/>
       <c r="R105" s="1139" t="n"/>
       <c r="S105" s="1139" t="n"/>
       <c r="T105" s="1139" t="n"/>
       <c r="U105" s="1157" t="n"/>
     </row>
-    <row r="106" ht="15" customHeight="1" s="1339">
-      <c r="A106" s="1340" t="n"/>
-      <c r="B106" s="1099" t="n"/>
-      <c r="C106" s="1099" t="n"/>
-      <c r="D106" s="1099" t="n"/>
-      <c r="E106" s="1099" t="n"/>
-      <c r="F106" s="1099" t="n"/>
-      <c r="G106" s="1099" t="n"/>
-      <c r="H106" s="1139" t="n"/>
-      <c r="I106" s="1139" t="n"/>
-      <c r="J106" s="1139" t="n"/>
-      <c r="K106" s="1139" t="n"/>
-      <c r="L106" s="1341" t="n"/>
-      <c r="M106" s="1099" t="n"/>
-      <c r="N106" s="1099" t="n"/>
-      <c r="O106" s="1099" t="n"/>
-      <c r="P106" s="1099" t="n"/>
+    <row r="106" ht="15" customFormat="1" customHeight="1" s="1073">
+      <c r="A106" s="1337" t="n"/>
+      <c r="B106" s="1177" t="n"/>
+      <c r="C106" s="1178" t="n"/>
+      <c r="D106" s="1233" t="n"/>
+      <c r="E106" s="1177" t="n"/>
+      <c r="F106" s="1177" t="n"/>
+      <c r="G106" s="1177" t="n"/>
+      <c r="H106" s="1177" t="n"/>
+      <c r="I106" s="1177" t="n"/>
+      <c r="J106" s="1177" t="n"/>
+      <c r="K106" s="1177" t="n"/>
+      <c r="L106" s="1177" t="n"/>
+      <c r="M106" s="1178" t="n"/>
+      <c r="N106" s="1338" t="n"/>
+      <c r="O106" s="1178" t="n"/>
+      <c r="P106" s="1337" t="n"/>
       <c r="Q106" s="1138" t="n"/>
       <c r="R106" s="1139" t="n"/>
       <c r="S106" s="1139" t="n"/>
       <c r="T106" s="1139" t="n"/>
       <c r="U106" s="1157" t="n"/>
     </row>
-    <row r="107" ht="15" customHeight="1" s="1339">
-      <c r="C107" s="1342" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="D107" s="1139" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="E107" s="1139" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="F107" s="1139" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="G107" s="1139" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="H107" s="1343" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="I107" s="1343" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="J107" s="1343" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="K107" s="1343" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="L107" s="1343" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="M107" s="1341" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="N107" s="1344" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="O107" s="1344" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="P107" s="1343" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
+    <row r="107" ht="15" customFormat="1" customHeight="1" s="1073">
+      <c r="A107" s="1305" t="n"/>
+      <c r="B107" s="1198" t="n"/>
+      <c r="C107" s="1199" t="n"/>
+      <c r="D107" s="1305" t="n"/>
+      <c r="E107" s="1198" t="n"/>
+      <c r="F107" s="1198" t="n"/>
+      <c r="G107" s="1198" t="n"/>
+      <c r="H107" s="1198" t="n"/>
+      <c r="I107" s="1198" t="n"/>
+      <c r="J107" s="1198" t="n"/>
+      <c r="K107" s="1198" t="n"/>
+      <c r="L107" s="1198" t="n"/>
+      <c r="M107" s="1198" t="n"/>
+      <c r="N107" s="1198" t="n"/>
+      <c r="O107" s="1198" t="n"/>
+      <c r="P107" s="1199" t="n"/>
       <c r="Q107" s="1138" t="n"/>
       <c r="R107" s="1139" t="n"/>
       <c r="S107" s="1139" t="n"/>
       <c r="T107" s="1139" t="n"/>
-      <c r="U107" s="1139" t="n"/>
-      <c r="V107" s="1343" t="n"/>
-      <c r="W107" s="1343" t="n"/>
-      <c r="X107" s="1343" t="n"/>
-      <c r="Y107" s="1343" t="n"/>
-      <c r="Z107" s="1343" t="n"/>
-      <c r="AA107" s="1343" t="n"/>
-      <c r="AB107" s="1343" t="n"/>
-      <c r="AC107" s="1343" t="n"/>
-      <c r="AD107" s="1343" t="n"/>
-      <c r="AE107" s="1343" t="n"/>
-      <c r="AF107" s="1343" t="n"/>
-      <c r="AG107" s="1343" t="n"/>
+      <c r="U107" s="1157" t="n"/>
+    </row>
+    <row r="108" ht="15" customHeight="1" s="1339">
+      <c r="A108" s="1340" t="n"/>
+      <c r="B108" s="1099" t="n"/>
+      <c r="C108" s="1099" t="n"/>
+      <c r="D108" s="1099" t="n"/>
+      <c r="E108" s="1099" t="n"/>
+      <c r="F108" s="1099" t="n"/>
+      <c r="G108" s="1099" t="n"/>
+      <c r="H108" s="1139" t="n"/>
+      <c r="I108" s="1139" t="n"/>
+      <c r="J108" s="1139" t="n"/>
+      <c r="K108" s="1139" t="n"/>
+      <c r="L108" s="1341" t="n"/>
+      <c r="M108" s="1099" t="n"/>
+      <c r="N108" s="1099" t="n"/>
+      <c r="O108" s="1099" t="n"/>
+      <c r="P108" s="1099" t="n"/>
+      <c r="Q108" s="1138" t="n"/>
+      <c r="R108" s="1139" t="n"/>
+      <c r="S108" s="1139" t="n"/>
+      <c r="T108" s="1139" t="n"/>
+      <c r="U108" s="1157" t="n"/>
+    </row>
+    <row r="109" ht="15" customHeight="1" s="1339">
+      <c r="C109" s="1342" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="D109" s="1139" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="E109" s="1139" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F109" s="1139" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="G109" s="1139" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="H109" s="1343" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="I109" s="1343" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="J109" s="1343" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="K109" s="1343" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="L109" s="1343" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="M109" s="1341" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="N109" s="1344" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="O109" s="1344" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="P109" s="1343" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="Q109" s="1138" t="n"/>
+      <c r="R109" s="1139" t="n"/>
+      <c r="S109" s="1139" t="n"/>
+      <c r="T109" s="1139" t="n"/>
+      <c r="U109" s="1139" t="n"/>
+      <c r="V109" s="1343" t="n"/>
+      <c r="W109" s="1343" t="n"/>
+      <c r="X109" s="1343" t="n"/>
+      <c r="Y109" s="1343" t="n"/>
+      <c r="Z109" s="1343" t="n"/>
+      <c r="AA109" s="1343" t="n"/>
+      <c r="AB109" s="1343" t="n"/>
+      <c r="AC109" s="1343" t="n"/>
+      <c r="AD109" s="1343" t="n"/>
+      <c r="AE109" s="1343" t="n"/>
+      <c r="AF109" s="1343" t="n"/>
+      <c r="AG109" s="1343" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="309">
-    <mergeCell ref="N101:O101"/>
+  <mergeCells count="317">
+    <mergeCell ref="N103:O103"/>
     <mergeCell ref="L50:O50"/>
-    <mergeCell ref="D102:M102"/>
-    <mergeCell ref="N100:O100"/>
+    <mergeCell ref="D104:M104"/>
+    <mergeCell ref="N102:O102"/>
     <mergeCell ref="G62:I62"/>
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="L52:O52"/>
@@ -13474,13 +13520,13 @@
     <mergeCell ref="A58:D58"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="I30:O30"/>
-    <mergeCell ref="L93:P93"/>
-    <mergeCell ref="A73:D73"/>
+    <mergeCell ref="L95:P95"/>
+    <mergeCell ref="A75:D75"/>
     <mergeCell ref="Q63:R63"/>
     <mergeCell ref="A60:D60"/>
     <mergeCell ref="A52:C52"/>
-    <mergeCell ref="E88:H88"/>
-    <mergeCell ref="E82:H82"/>
+    <mergeCell ref="E90:H90"/>
+    <mergeCell ref="E84:H84"/>
     <mergeCell ref="A34:C34"/>
     <mergeCell ref="L45:O45"/>
     <mergeCell ref="A49:C49"/>
@@ -13492,25 +13538,25 @@
     <mergeCell ref="A55:C55"/>
     <mergeCell ref="E48:F48"/>
     <mergeCell ref="G48:H48"/>
-    <mergeCell ref="E75:H75"/>
+    <mergeCell ref="E77:H77"/>
     <mergeCell ref="I54:J54"/>
     <mergeCell ref="G12:J12"/>
-    <mergeCell ref="A83:P83"/>
-    <mergeCell ref="N102:O102"/>
+    <mergeCell ref="A85:P85"/>
+    <mergeCell ref="N104:O104"/>
     <mergeCell ref="A29:C29"/>
     <mergeCell ref="I56:J56"/>
     <mergeCell ref="I43:J43"/>
-    <mergeCell ref="A79:D79"/>
+    <mergeCell ref="A81:D81"/>
     <mergeCell ref="A44:C44"/>
     <mergeCell ref="I70:L70"/>
     <mergeCell ref="A31:C31"/>
     <mergeCell ref="N17:P20"/>
     <mergeCell ref="A24:C24"/>
     <mergeCell ref="A65:P65"/>
-    <mergeCell ref="A74:D74"/>
-    <mergeCell ref="E90:H90"/>
     <mergeCell ref="A76:D76"/>
-    <mergeCell ref="I75:K75"/>
+    <mergeCell ref="E92:H92"/>
+    <mergeCell ref="A78:D78"/>
+    <mergeCell ref="I77:K77"/>
     <mergeCell ref="L59:O59"/>
     <mergeCell ref="L46:O46"/>
     <mergeCell ref="G25:J25"/>
@@ -13520,65 +13566,65 @@
     <mergeCell ref="G58:I58"/>
     <mergeCell ref="L61:O61"/>
     <mergeCell ref="L48:O48"/>
-    <mergeCell ref="A92:D92"/>
+    <mergeCell ref="A94:D94"/>
     <mergeCell ref="A69:D69"/>
     <mergeCell ref="L43:O43"/>
     <mergeCell ref="G13:J13"/>
     <mergeCell ref="G51:H51"/>
-    <mergeCell ref="E78:H78"/>
+    <mergeCell ref="E80:H80"/>
     <mergeCell ref="I51:J51"/>
-    <mergeCell ref="A89:D89"/>
+    <mergeCell ref="A91:D91"/>
     <mergeCell ref="G15:J15"/>
-    <mergeCell ref="E80:H80"/>
+    <mergeCell ref="E82:H82"/>
     <mergeCell ref="I39:O39"/>
-    <mergeCell ref="L82:P82"/>
+    <mergeCell ref="L84:P84"/>
     <mergeCell ref="E42:F42"/>
-    <mergeCell ref="E81:H81"/>
-    <mergeCell ref="L75:P75"/>
+    <mergeCell ref="E83:H83"/>
+    <mergeCell ref="L77:P77"/>
     <mergeCell ref="M66:P66"/>
-    <mergeCell ref="A82:D82"/>
+    <mergeCell ref="A84:D84"/>
     <mergeCell ref="G60:I60"/>
-    <mergeCell ref="A85:E85"/>
+    <mergeCell ref="A87:E87"/>
     <mergeCell ref="L62:O62"/>
     <mergeCell ref="A66:D66"/>
-    <mergeCell ref="A99:P99"/>
+    <mergeCell ref="A101:P101"/>
     <mergeCell ref="N16:P16"/>
     <mergeCell ref="A45:C45"/>
-    <mergeCell ref="L72:P72"/>
+    <mergeCell ref="L74:P74"/>
     <mergeCell ref="L51:O51"/>
     <mergeCell ref="I67:L67"/>
     <mergeCell ref="E47:F47"/>
     <mergeCell ref="K7:M8"/>
     <mergeCell ref="A46:C46"/>
-    <mergeCell ref="A72:D72"/>
-    <mergeCell ref="A105:C105"/>
+    <mergeCell ref="A74:D74"/>
+    <mergeCell ref="A107:C107"/>
     <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A86:F86"/>
+    <mergeCell ref="A88:F88"/>
     <mergeCell ref="E63:F63"/>
-    <mergeCell ref="I79:K79"/>
-    <mergeCell ref="I73:K73"/>
-    <mergeCell ref="L85:P85"/>
-    <mergeCell ref="I74:K74"/>
+    <mergeCell ref="I81:K81"/>
+    <mergeCell ref="I75:K75"/>
+    <mergeCell ref="L87:P87"/>
+    <mergeCell ref="I76:K76"/>
     <mergeCell ref="N4:P4"/>
-    <mergeCell ref="L84:P84"/>
-    <mergeCell ref="L80:P80"/>
+    <mergeCell ref="L86:P86"/>
+    <mergeCell ref="L82:P82"/>
     <mergeCell ref="I33:O33"/>
-    <mergeCell ref="A71:P71"/>
+    <mergeCell ref="A73:P73"/>
     <mergeCell ref="I35:O35"/>
-    <mergeCell ref="I92:K92"/>
+    <mergeCell ref="I94:K94"/>
     <mergeCell ref="C7:D8"/>
     <mergeCell ref="A32:C32"/>
     <mergeCell ref="E7:F8"/>
-    <mergeCell ref="L73:P73"/>
-    <mergeCell ref="I81:K81"/>
-    <mergeCell ref="I76:K76"/>
+    <mergeCell ref="L75:P75"/>
+    <mergeCell ref="I83:K83"/>
+    <mergeCell ref="I78:K78"/>
     <mergeCell ref="A16:C16"/>
-    <mergeCell ref="L86:P86"/>
+    <mergeCell ref="L88:P88"/>
     <mergeCell ref="G26:J26"/>
-    <mergeCell ref="A91:D91"/>
+    <mergeCell ref="A93:D93"/>
     <mergeCell ref="A1:P2"/>
     <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A93:D93"/>
+    <mergeCell ref="A95:D95"/>
     <mergeCell ref="A68:D68"/>
     <mergeCell ref="A19:M19"/>
     <mergeCell ref="A47:C47"/>
@@ -13587,13 +13633,13 @@
     <mergeCell ref="E59:F59"/>
     <mergeCell ref="I36:O36"/>
     <mergeCell ref="E46:F46"/>
-    <mergeCell ref="D105:P105"/>
+    <mergeCell ref="D107:P107"/>
     <mergeCell ref="E61:F61"/>
-    <mergeCell ref="I89:K89"/>
+    <mergeCell ref="I91:K91"/>
     <mergeCell ref="E54:F54"/>
     <mergeCell ref="G54:H54"/>
     <mergeCell ref="E56:F56"/>
-    <mergeCell ref="D103:M103"/>
+    <mergeCell ref="D105:M105"/>
     <mergeCell ref="G56:H56"/>
     <mergeCell ref="E43:F43"/>
     <mergeCell ref="G43:H43"/>
@@ -13605,8 +13651,8 @@
     <mergeCell ref="A53:C53"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="G27:J27"/>
-    <mergeCell ref="L92:P92"/>
-    <mergeCell ref="A98:P98"/>
+    <mergeCell ref="L94:P94"/>
+    <mergeCell ref="A100:P100"/>
     <mergeCell ref="A48:C48"/>
     <mergeCell ref="H7:J8"/>
     <mergeCell ref="G29:H29"/>
@@ -13623,18 +13669,18 @@
     <mergeCell ref="A64:D64"/>
     <mergeCell ref="A43:C43"/>
     <mergeCell ref="G63:I63"/>
-    <mergeCell ref="E79:H79"/>
+    <mergeCell ref="E81:H81"/>
     <mergeCell ref="I42:J42"/>
     <mergeCell ref="K58:K63"/>
     <mergeCell ref="M70:P70"/>
-    <mergeCell ref="E73:H73"/>
+    <mergeCell ref="E75:H75"/>
     <mergeCell ref="I52:J52"/>
     <mergeCell ref="I32:O32"/>
     <mergeCell ref="N40:O40"/>
     <mergeCell ref="I44:J44"/>
     <mergeCell ref="I66:L66"/>
     <mergeCell ref="K9:M9"/>
-    <mergeCell ref="E74:H74"/>
+    <mergeCell ref="E76:H76"/>
     <mergeCell ref="I68:L68"/>
     <mergeCell ref="A62:D62"/>
     <mergeCell ref="R3:U14"/>
@@ -13646,119 +13692,119 @@
     <mergeCell ref="L57:O57"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A61:D61"/>
-    <mergeCell ref="A88:D88"/>
-    <mergeCell ref="A94:P94"/>
+    <mergeCell ref="A90:D90"/>
+    <mergeCell ref="A96:P96"/>
     <mergeCell ref="A40:C40"/>
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="L42:O42"/>
-    <mergeCell ref="A87:P87"/>
-    <mergeCell ref="A90:D90"/>
+    <mergeCell ref="A89:P89"/>
+    <mergeCell ref="A92:D92"/>
     <mergeCell ref="A51:C51"/>
     <mergeCell ref="E58:F58"/>
-    <mergeCell ref="N104:O104"/>
+    <mergeCell ref="N106:O106"/>
     <mergeCell ref="I45:J45"/>
-    <mergeCell ref="E76:H76"/>
-    <mergeCell ref="L78:P78"/>
+    <mergeCell ref="E78:H78"/>
+    <mergeCell ref="L80:P80"/>
     <mergeCell ref="I47:J47"/>
     <mergeCell ref="N23:P25"/>
     <mergeCell ref="I69:L69"/>
-    <mergeCell ref="A84:E84"/>
+    <mergeCell ref="A86:E86"/>
     <mergeCell ref="G11:J11"/>
     <mergeCell ref="A5:D6"/>
     <mergeCell ref="L47:O47"/>
-    <mergeCell ref="E92:H92"/>
-    <mergeCell ref="A78:D78"/>
+    <mergeCell ref="E94:H94"/>
+    <mergeCell ref="A80:D80"/>
     <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A80:D80"/>
+    <mergeCell ref="A82:D82"/>
     <mergeCell ref="A7:B8"/>
     <mergeCell ref="L58:O58"/>
-    <mergeCell ref="E89:H89"/>
+    <mergeCell ref="E91:H91"/>
     <mergeCell ref="A54:C54"/>
     <mergeCell ref="L60:O60"/>
     <mergeCell ref="G64:J64"/>
     <mergeCell ref="A56:C56"/>
     <mergeCell ref="A27:C27"/>
-    <mergeCell ref="E72:H72"/>
+    <mergeCell ref="E74:H74"/>
     <mergeCell ref="K3:M4"/>
     <mergeCell ref="G53:H53"/>
     <mergeCell ref="I53:J53"/>
     <mergeCell ref="I55:J55"/>
-    <mergeCell ref="L79:P79"/>
+    <mergeCell ref="L81:P81"/>
     <mergeCell ref="I48:J48"/>
     <mergeCell ref="A41:P41"/>
-    <mergeCell ref="I77:K77"/>
-    <mergeCell ref="A75:D75"/>
+    <mergeCell ref="I79:K79"/>
+    <mergeCell ref="A77:D77"/>
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="A11:C11"/>
-    <mergeCell ref="L81:P81"/>
-    <mergeCell ref="G84:K84"/>
+    <mergeCell ref="L83:P83"/>
+    <mergeCell ref="G86:K86"/>
     <mergeCell ref="M64:O64"/>
     <mergeCell ref="G14:J14"/>
-    <mergeCell ref="I72:K72"/>
-    <mergeCell ref="A81:D81"/>
-    <mergeCell ref="I88:K88"/>
-    <mergeCell ref="L74:P74"/>
-    <mergeCell ref="I82:K82"/>
+    <mergeCell ref="I74:K74"/>
+    <mergeCell ref="A83:D83"/>
+    <mergeCell ref="I90:K90"/>
+    <mergeCell ref="L76:P76"/>
+    <mergeCell ref="I84:K84"/>
     <mergeCell ref="L53:O53"/>
     <mergeCell ref="A70:D70"/>
-    <mergeCell ref="L76:P76"/>
+    <mergeCell ref="L78:P78"/>
     <mergeCell ref="E49:F49"/>
-    <mergeCell ref="N103:O103"/>
+    <mergeCell ref="N105:O105"/>
     <mergeCell ref="Q1:U2"/>
     <mergeCell ref="G44:H44"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A3:B4"/>
-    <mergeCell ref="E91:H91"/>
+    <mergeCell ref="E93:H93"/>
     <mergeCell ref="G20:J20"/>
-    <mergeCell ref="G85:J85"/>
+    <mergeCell ref="G87:J87"/>
     <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A104:C104"/>
-    <mergeCell ref="E93:H93"/>
+    <mergeCell ref="A106:C106"/>
+    <mergeCell ref="E95:H95"/>
     <mergeCell ref="A14:C14"/>
-    <mergeCell ref="G86:J86"/>
-    <mergeCell ref="L89:P89"/>
-    <mergeCell ref="I78:K78"/>
+    <mergeCell ref="G88:J88"/>
+    <mergeCell ref="L91:P91"/>
+    <mergeCell ref="I80:K80"/>
     <mergeCell ref="G49:H49"/>
-    <mergeCell ref="L88:P88"/>
-    <mergeCell ref="D104:M104"/>
-    <mergeCell ref="I90:K90"/>
+    <mergeCell ref="L90:P90"/>
+    <mergeCell ref="D106:M106"/>
+    <mergeCell ref="I92:K92"/>
     <mergeCell ref="I37:O37"/>
-    <mergeCell ref="I91:K91"/>
+    <mergeCell ref="I93:K93"/>
     <mergeCell ref="N21:P21"/>
-    <mergeCell ref="L77:P77"/>
+    <mergeCell ref="L79:P79"/>
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="E50:F50"/>
     <mergeCell ref="L44:O44"/>
     <mergeCell ref="G42:H42"/>
-    <mergeCell ref="I93:K93"/>
-    <mergeCell ref="A101:C101"/>
+    <mergeCell ref="I95:K95"/>
+    <mergeCell ref="A103:C103"/>
     <mergeCell ref="E52:F52"/>
     <mergeCell ref="A10:M10"/>
     <mergeCell ref="E44:F44"/>
     <mergeCell ref="E66:H66"/>
-    <mergeCell ref="A77:D77"/>
+    <mergeCell ref="A79:D79"/>
     <mergeCell ref="M68:P68"/>
     <mergeCell ref="E68:H68"/>
     <mergeCell ref="A20:C20"/>
     <mergeCell ref="M67:P67"/>
     <mergeCell ref="C3:G4"/>
-    <mergeCell ref="D101:M101"/>
+    <mergeCell ref="D103:M103"/>
     <mergeCell ref="M69:P69"/>
     <mergeCell ref="E57:F57"/>
-    <mergeCell ref="I80:K80"/>
-    <mergeCell ref="L90:P90"/>
+    <mergeCell ref="I82:K82"/>
+    <mergeCell ref="L92:P92"/>
     <mergeCell ref="G50:H50"/>
     <mergeCell ref="I50:J50"/>
     <mergeCell ref="H3:J4"/>
     <mergeCell ref="G52:H52"/>
-    <mergeCell ref="L91:P91"/>
+    <mergeCell ref="L93:P93"/>
     <mergeCell ref="I38:O38"/>
     <mergeCell ref="A33:C33"/>
     <mergeCell ref="E5:M6"/>
-    <mergeCell ref="A100:C100"/>
+    <mergeCell ref="A102:C102"/>
     <mergeCell ref="A35:C35"/>
     <mergeCell ref="E60:F60"/>
-    <mergeCell ref="A102:C102"/>
+    <mergeCell ref="A104:C104"/>
     <mergeCell ref="E45:F45"/>
     <mergeCell ref="G45:H45"/>
     <mergeCell ref="A39:C39"/>
@@ -13766,11 +13812,19 @@
     <mergeCell ref="G55:H55"/>
     <mergeCell ref="E69:H69"/>
     <mergeCell ref="G47:H47"/>
-    <mergeCell ref="A103:C103"/>
+    <mergeCell ref="A105:C105"/>
     <mergeCell ref="G61:I61"/>
     <mergeCell ref="G46:H46"/>
-    <mergeCell ref="E77:H77"/>
+    <mergeCell ref="E79:H79"/>
     <mergeCell ref="L63:O63"/>
+    <mergeCell ref="I71:L71"/>
+    <mergeCell ref="E71:H71"/>
+    <mergeCell ref="M71:P71"/>
+    <mergeCell ref="A71:D71"/>
+    <mergeCell ref="I72:L72"/>
+    <mergeCell ref="E72:H72"/>
+    <mergeCell ref="M72:P72"/>
+    <mergeCell ref="A72:D72"/>
   </mergeCells>
   <conditionalFormatting sqref="M26">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="lessThan" aboveAverage="0" dxfId="0" text="" percent="0" bottom="0">
@@ -15568,18 +15622,18 @@
         </is>
       </c>
       <c r="I25" s="1479">
-        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A73="","",'Recept-voorblad'!A73),IF('Recept-voorblad'!A89="-","-",IF('Recept-voorblad'!A89="Revisie nummer","",'Recept-voorblad'!A89)))</f>
+        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A75="","",'Recept-voorblad'!A75),IF('Recept-voorblad'!A91="-","-",IF('Recept-voorblad'!A91="Revisie nummer","",'Recept-voorblad'!A91)))</f>
         <v/>
       </c>
       <c r="J25" s="1223" t="n"/>
       <c r="K25" s="1224" t="n"/>
       <c r="L25" s="1480">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E73="","",'Recept-voorblad'!E73),IF('Recept-voorblad'!E89="","",'Recept-voorblad'!E89))</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E75="","",'Recept-voorblad'!E75),IF('Recept-voorblad'!E91="","",'Recept-voorblad'!E91))</f>
         <v/>
       </c>
       <c r="M25" s="1481" t="n"/>
       <c r="N25" s="1482">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I73="","",'Recept-voorblad'!I73),IF('Recept-voorblad'!I89="","",'Recept-voorblad'!I89))</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I75="","",'Recept-voorblad'!I75),IF('Recept-voorblad'!I91="","",'Recept-voorblad'!I91))</f>
         <v/>
       </c>
       <c r="O25" s="1481" t="n"/>
@@ -15670,18 +15724,18 @@
         </is>
       </c>
       <c r="I26" s="1486">
-        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A74="","",'Recept-voorblad'!A74),IF('Recept-voorblad'!A90="-","-",IF('Recept-voorblad'!A90="Revisie nummer","",'Recept-voorblad'!A90)))</f>
+        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A76="","",'Recept-voorblad'!A76),IF('Recept-voorblad'!A92="-","-",IF('Recept-voorblad'!A92="Revisie nummer","",'Recept-voorblad'!A92)))</f>
         <v/>
       </c>
       <c r="J26" s="1177" t="n"/>
       <c r="K26" s="1178" t="n"/>
       <c r="L26" s="1487">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E74="","",'Recept-voorblad'!E74),IF('Recept-voorblad'!E90="","",'Recept-voorblad'!E90))</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E76="","",'Recept-voorblad'!E76),IF('Recept-voorblad'!E92="","",'Recept-voorblad'!E92))</f>
         <v/>
       </c>
       <c r="M26" s="1488" t="n"/>
       <c r="N26" s="1489">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I74="","",'Recept-voorblad'!I74),IF('Recept-voorblad'!I90="","",'Recept-voorblad'!I90))</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I76="","",'Recept-voorblad'!I76),IF('Recept-voorblad'!I92="","",'Recept-voorblad'!I92))</f>
         <v/>
       </c>
       <c r="O26" s="1488" t="n"/>
@@ -15760,18 +15814,18 @@
         </is>
       </c>
       <c r="I27" s="1486">
-        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A75="","",'Recept-voorblad'!A75),IF('Recept-voorblad'!A91="-","-",IF('Recept-voorblad'!A91="Revisie nummer","",'Recept-voorblad'!A91)))</f>
+        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A77="","",'Recept-voorblad'!A77),IF('Recept-voorblad'!A93="-","-",IF('Recept-voorblad'!A93="Revisie nummer","",'Recept-voorblad'!A93)))</f>
         <v/>
       </c>
       <c r="J27" s="1177" t="n"/>
       <c r="K27" s="1178" t="n"/>
       <c r="L27" s="1487">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E75="","",'Recept-voorblad'!E75),IF('Recept-voorblad'!E91="","",'Recept-voorblad'!E91))</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E77="","",'Recept-voorblad'!E77),IF('Recept-voorblad'!E93="","",'Recept-voorblad'!E93))</f>
         <v/>
       </c>
       <c r="M27" s="1488" t="n"/>
       <c r="N27" s="1489">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I75="","",'Recept-voorblad'!I75),IF('Recept-voorblad'!I91="","",'Recept-voorblad'!I91))</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I77="","",'Recept-voorblad'!I77),IF('Recept-voorblad'!I93="","",'Recept-voorblad'!I93))</f>
         <v/>
       </c>
       <c r="O27" s="1488" t="n"/>
@@ -15822,18 +15876,18 @@
         </is>
       </c>
       <c r="I28" s="1486">
-        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A76="","",'Recept-voorblad'!A76),IF('Recept-voorblad'!A92="-","-",IF('Recept-voorblad'!A92="Revisie nummer","",'Recept-voorblad'!A92)))</f>
+        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A78="","",'Recept-voorblad'!A78),IF('Recept-voorblad'!A94="-","-",IF('Recept-voorblad'!A94="Revisie nummer","",'Recept-voorblad'!A94)))</f>
         <v/>
       </c>
       <c r="J28" s="1177" t="n"/>
       <c r="K28" s="1178" t="n"/>
       <c r="L28" s="1487">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E76="","",'Recept-voorblad'!E76),IF('Recept-voorblad'!E92="","",'Recept-voorblad'!E92))</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E78="","",'Recept-voorblad'!E78),IF('Recept-voorblad'!E94="","",'Recept-voorblad'!E94))</f>
         <v/>
       </c>
       <c r="M28" s="1488" t="n"/>
       <c r="N28" s="1489">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I76="","",'Recept-voorblad'!I76),IF('Recept-voorblad'!I92="","",'Recept-voorblad'!I92))</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I78="","",'Recept-voorblad'!I78),IF('Recept-voorblad'!I94="","",'Recept-voorblad'!I94))</f>
         <v/>
       </c>
       <c r="O28" s="1488" t="n"/>
@@ -15920,18 +15974,18 @@
         </is>
       </c>
       <c r="I29" s="1486">
-        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A77="","",'Recept-voorblad'!A77),IF('Recept-voorblad'!A93="-","-",IF('Recept-voorblad'!A93="Revisie nummer","",'Recept-voorblad'!A93)))</f>
+        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A79="","",'Recept-voorblad'!A79),IF('Recept-voorblad'!A95="-","-",IF('Recept-voorblad'!A95="Revisie nummer","",'Recept-voorblad'!A95)))</f>
         <v/>
       </c>
       <c r="J29" s="1177" t="n"/>
       <c r="K29" s="1178" t="n"/>
       <c r="L29" s="1487">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E77="","",'Recept-voorblad'!E77),IF('Recept-voorblad'!E93="","",'Recept-voorblad'!E93))</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E79="","",'Recept-voorblad'!E79),IF('Recept-voorblad'!E95="","",'Recept-voorblad'!E95))</f>
         <v/>
       </c>
       <c r="M29" s="1488" t="n"/>
       <c r="N29" s="1489">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I77="","",'Recept-voorblad'!I77),IF('Recept-voorblad'!I93="","",'Recept-voorblad'!I93))</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I79="","",'Recept-voorblad'!I79),IF('Recept-voorblad'!I95="","",'Recept-voorblad'!I95))</f>
         <v/>
       </c>
       <c r="O29" s="1488" t="n"/>
@@ -16035,18 +16089,18 @@
       <c r="G30" s="1089" t="n"/>
       <c r="H30" s="1090" t="n"/>
       <c r="I30" s="1513">
-        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A78="","",'Recept-voorblad'!A78),"-")</f>
+        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A80="","",'Recept-voorblad'!A80),"-")</f>
         <v/>
       </c>
       <c r="J30" s="1177" t="n"/>
       <c r="K30" s="1178" t="n"/>
       <c r="L30" s="1487">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E78="","",'Recept-voorblad'!E78),"-")</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E80="","",'Recept-voorblad'!E80),"-")</f>
         <v/>
       </c>
       <c r="M30" s="1488" t="n"/>
       <c r="N30" s="1489">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I78="","",'Recept-voorblad'!I78),"-")</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I80="","",'Recept-voorblad'!I80),"-")</f>
         <v/>
       </c>
       <c r="O30" s="1488" t="n"/>
@@ -16084,18 +16138,18 @@
       <c r="F31" s="1521" t="n"/>
       <c r="H31" s="1100" t="n"/>
       <c r="I31" s="1513">
-        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A79="","",'Recept-voorblad'!A79),"-")</f>
+        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A81="","",'Recept-voorblad'!A81),"-")</f>
         <v/>
       </c>
       <c r="J31" s="1177" t="n"/>
       <c r="K31" s="1178" t="n"/>
       <c r="L31" s="1487">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E79="","",'Recept-voorblad'!E79),"-")</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E81="","",'Recept-voorblad'!E81),"-")</f>
         <v/>
       </c>
       <c r="M31" s="1488" t="n"/>
       <c r="N31" s="1489">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I79="","",'Recept-voorblad'!I79),"-")</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I81="","",'Recept-voorblad'!I81),"-")</f>
         <v/>
       </c>
       <c r="O31" s="1488" t="n"/>
@@ -16169,18 +16223,18 @@
       <c r="F32" s="1521" t="n"/>
       <c r="H32" s="1100" t="n"/>
       <c r="I32" s="1513">
-        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A80="","",'Recept-voorblad'!A80),"-")</f>
+        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A82="","",'Recept-voorblad'!A82),"-")</f>
         <v/>
       </c>
       <c r="J32" s="1177" t="n"/>
       <c r="K32" s="1178" t="n"/>
       <c r="L32" s="1487">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E80="","",'Recept-voorblad'!E80),"-")</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E82="","",'Recept-voorblad'!E82),"-")</f>
         <v/>
       </c>
       <c r="M32" s="1488" t="n"/>
       <c r="N32" s="1489">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I80="","",'Recept-voorblad'!I80),"-")</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I82="","",'Recept-voorblad'!I82),"-")</f>
         <v/>
       </c>
       <c r="O32" s="1488" t="n"/>
@@ -16218,18 +16272,18 @@
       <c r="F33" s="1521" t="n"/>
       <c r="H33" s="1100" t="n"/>
       <c r="I33" s="1513">
-        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A81="","",'Recept-voorblad'!A81),"-")</f>
+        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A83="","",'Recept-voorblad'!A83),"-")</f>
         <v/>
       </c>
       <c r="J33" s="1177" t="n"/>
       <c r="K33" s="1178" t="n"/>
       <c r="L33" s="1487">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E81="","",'Recept-voorblad'!E81),"-")</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E83="","",'Recept-voorblad'!E83),"-")</f>
         <v/>
       </c>
       <c r="M33" s="1488" t="n"/>
       <c r="N33" s="1489">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I81="","",'Recept-voorblad'!I81),"-")</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I83="","",'Recept-voorblad'!I83),"-")</f>
         <v/>
       </c>
       <c r="O33" s="1488" t="n"/>
@@ -16309,18 +16363,18 @@
       <c r="G34" s="1168" t="n"/>
       <c r="H34" s="1169" t="n"/>
       <c r="I34" s="1532">
-        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A82="","",'Recept-voorblad'!A82),"-")</f>
+        <f>IF(LEFT(A1,2)="WP",IF('Recept-voorblad'!A84="","",'Recept-voorblad'!A84),"-")</f>
         <v/>
       </c>
       <c r="J34" s="1507" t="n"/>
       <c r="K34" s="1533" t="n"/>
       <c r="L34" s="1534">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E82="","",'Recept-voorblad'!E82),"-")</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!E84="","",'Recept-voorblad'!E84),"-")</f>
         <v/>
       </c>
       <c r="M34" s="1535" t="n"/>
       <c r="N34" s="1536">
-        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I82="","",'Recept-voorblad'!I82),"-")</f>
+        <f>IF(LEFT($A$1,2)="WP",IF('Recept-voorblad'!I84="","",'Recept-voorblad'!I84),"-")</f>
         <v/>
       </c>
       <c r="O34" s="1535" t="n"/>
@@ -16477,7 +16531,7 @@
         <v/>
       </c>
       <c r="I36" s="1547">
-        <f>IF(LEFT(A1,2)="WP","Inmaischen",'Recept-voorblad'!A73)</f>
+        <f>IF(LEFT(A1,2)="WP","Inmaischen",'Recept-voorblad'!A75)</f>
         <v/>
       </c>
       <c r="J36" s="1075" t="n"/>
@@ -16577,7 +16631,7 @@
         <v/>
       </c>
       <c r="I37" s="1559">
-        <f>IF(LEFT(A1,2)="WP", "Koken",'Recept-voorblad'!A74)</f>
+        <f>IF(LEFT(A1,2)="WP", "Koken",'Recept-voorblad'!A76)</f>
         <v/>
       </c>
       <c r="L37" s="1560">
@@ -16666,7 +16720,7 @@
         <v/>
       </c>
       <c r="I38" s="1568">
-        <f>IF(LEFT(A1,2)="WP", "Inline sparge",'Recept-voorblad'!A75)</f>
+        <f>IF(LEFT(A1,2)="WP", "Inline sparge",'Recept-voorblad'!A77)</f>
         <v/>
       </c>
       <c r="L38" s="1083" t="n"/>
@@ -16761,12 +16815,12 @@
         <v/>
       </c>
       <c r="I39" s="1568">
-        <f>IF(LEFT(A1,2)="WP", " ",'Recept-voorblad'!A76)</f>
+        <f>IF(LEFT(A1,2)="WP", " ",'Recept-voorblad'!A78)</f>
         <v/>
       </c>
       <c r="L39" s="1083" t="n"/>
       <c r="M39" s="1561">
-        <f>IF(LEFT(A1,2)="WP"," ",'Recept-voorblad'!E76&amp;" "&amp;'Recept-voorblad'!I76)</f>
+        <f>IF(LEFT(A1,2)="WP"," ",'Recept-voorblad'!E78&amp;" "&amp;'Recept-voorblad'!I78)</f>
         <v/>
       </c>
       <c r="N39" s="1561" t="n"/>
@@ -16886,12 +16940,12 @@
         <v/>
       </c>
       <c r="I40" s="1568">
-        <f>IF(LEFT(A1,2)="WP", " ",'Recept-voorblad'!A77)</f>
+        <f>IF(LEFT(A1,2)="WP", " ",'Recept-voorblad'!A79)</f>
         <v/>
       </c>
       <c r="L40" s="1083" t="n"/>
       <c r="M40" s="1561">
-        <f>IF(LEFT(A1,2)="WP"," ",'Recept-voorblad'!E77&amp;" "&amp;'Recept-voorblad'!I77)</f>
+        <f>IF(LEFT(A1,2)="WP"," ",'Recept-voorblad'!E79&amp;" "&amp;'Recept-voorblad'!I79)</f>
         <v/>
       </c>
       <c r="N40" s="1561" t="n"/>
@@ -17014,12 +17068,12 @@
         <v/>
       </c>
       <c r="I41" s="1568">
-        <f>IF(LEFT(A1,2)="WP", " ",'Recept-voorblad'!A78)</f>
+        <f>IF(LEFT(A1,2)="WP", " ",'Recept-voorblad'!A80)</f>
         <v/>
       </c>
       <c r="L41" s="1083" t="n"/>
       <c r="M41" s="1561">
-        <f>IF(LEFT(A1,2)="WP"," ",'Recept-voorblad'!E78&amp;" "&amp;'Recept-voorblad'!I78)</f>
+        <f>IF(LEFT(A1,2)="WP"," ",'Recept-voorblad'!E80&amp;" "&amp;'Recept-voorblad'!I80)</f>
         <v/>
       </c>
       <c r="N41" s="1561" t="n"/>
@@ -17466,7 +17520,7 @@
       </c>
       <c r="M46" s="1083" t="n"/>
       <c r="N46" s="1609">
-        <f>SUBSTITUTE('Recept-voorblad'!A85&amp;IF('Recept-voorblad'!A86=0,"",'Recept-voorblad'!A86),"(g/brew)"," ")</f>
+        <f>SUBSTITUTE('Recept-voorblad'!A87&amp;IF('Recept-voorblad'!A88=0,"",'Recept-voorblad'!A88),"(g/brew)"," ")</f>
         <v/>
       </c>
       <c r="O46" s="1178" t="n"/>
@@ -17557,7 +17611,7 @@
       </c>
       <c r="M48" s="1083" t="n"/>
       <c r="N48" s="1617">
-        <f>'Recept-voorblad'!G85+IF('Recept-voorblad'!G86="",0,'Recept-voorblad'!G86)</f>
+        <f>'Recept-voorblad'!G87+IF('Recept-voorblad'!G88="",0,'Recept-voorblad'!G88)</f>
         <v/>
       </c>
       <c r="O48" s="1178" t="n"/>
@@ -21211,7 +21265,7 @@
       <c r="M23" s="1747" t="n"/>
       <c r="N23" s="1748" t="n"/>
       <c r="O23" s="1739">
-        <f>IF('Recept-voorblad'!I89="-","-",'Recept-voorblad'!E89&amp;" "&amp;'Recept-voorblad'!A89&amp;" @"&amp;'Recept-voorblad'!I89)</f>
+        <f>IF('Recept-voorblad'!I91="-","-",'Recept-voorblad'!E91&amp;" "&amp;'Recept-voorblad'!A91&amp;" @"&amp;'Recept-voorblad'!I91)</f>
         <v/>
       </c>
       <c r="P23" s="1747" t="n"/>
@@ -21253,7 +21307,7 @@
       <c r="M24" s="1747" t="n"/>
       <c r="N24" s="1748" t="n"/>
       <c r="O24" s="1739">
-        <f>IF('Recept-voorblad'!I90="-","-",'Recept-voorblad'!E90&amp;" "&amp;'Recept-voorblad'!A90&amp;" @"&amp;'Recept-voorblad'!I90)</f>
+        <f>IF('Recept-voorblad'!I92="-","-",'Recept-voorblad'!E92&amp;" "&amp;'Recept-voorblad'!A92&amp;" @"&amp;'Recept-voorblad'!I92)</f>
         <v/>
       </c>
       <c r="P24" s="1747" t="n"/>
@@ -21295,7 +21349,7 @@
       <c r="M25" s="1747" t="n"/>
       <c r="N25" s="1748" t="n"/>
       <c r="O25" s="1739">
-        <f>IF('Recept-voorblad'!I91="-","-",'Recept-voorblad'!E91&amp;" "&amp;'Recept-voorblad'!A91&amp;" @"&amp;'Recept-voorblad'!I91)</f>
+        <f>IF('Recept-voorblad'!I93="-","-",'Recept-voorblad'!E93&amp;" "&amp;'Recept-voorblad'!A93&amp;" @"&amp;'Recept-voorblad'!I93)</f>
         <v/>
       </c>
       <c r="P25" s="1747" t="n"/>
@@ -21337,7 +21391,7 @@
       <c r="M26" s="1747" t="n"/>
       <c r="N26" s="1748" t="n"/>
       <c r="O26" s="1739">
-        <f>IF('Recept-voorblad'!I92="-","-",'Recept-voorblad'!E92&amp;" "&amp;'Recept-voorblad'!A92&amp;" @"&amp;'Recept-voorblad'!I92)</f>
+        <f>IF('Recept-voorblad'!I94="-","-",'Recept-voorblad'!E94&amp;" "&amp;'Recept-voorblad'!A94&amp;" @"&amp;'Recept-voorblad'!I94)</f>
         <v/>
       </c>
       <c r="P26" s="1747" t="n"/>
@@ -21376,7 +21430,7 @@
       <c r="M27" s="1747" t="n"/>
       <c r="N27" s="1748" t="n"/>
       <c r="O27" s="1739">
-        <f>IF('Recept-voorblad'!I93="-","-",'Recept-voorblad'!E93&amp;" "&amp;'Recept-voorblad'!A93&amp;" @"&amp;'Recept-voorblad'!I93)</f>
+        <f>IF('Recept-voorblad'!I95="-","-",'Recept-voorblad'!E95&amp;" "&amp;'Recept-voorblad'!A95&amp;" @"&amp;'Recept-voorblad'!I95)</f>
         <v/>
       </c>
       <c r="P27" s="1747" t="n"/>
@@ -22508,7 +22562,7 @@
       <c r="Y54" s="1159" t="n"/>
       <c r="Z54" s="1761" t="n"/>
       <c r="AA54" s="1764">
-        <f>VLOOKUP("*Nagardo*",'Recept-voorblad'!A89:H93,5,FALSE())</f>
+        <f>VLOOKUP("*Nagardo*",'Recept-voorblad'!A91:H93,5,FALSE())</f>
         <v/>
       </c>
       <c r="AB54" s="1159" t="inlineStr">
@@ -22821,7 +22875,7 @@
       <c r="Y60" s="1602" t="n"/>
       <c r="Z60" s="1763" t="n"/>
       <c r="AA60" s="1763">
-        <f>'Recept-voorblad'!E90*(AA53/100)</f>
+        <f>'Recept-voorblad'!E92*(AA53/100)</f>
         <v/>
       </c>
       <c r="AB60" s="1159" t="inlineStr">
@@ -25279,7 +25333,7 @@
       <c r="T36" s="1602" t="n"/>
       <c r="U36" s="1939" t="n"/>
       <c r="V36" s="1763">
-        <f>VLOOKUP("*Nagardo*",'Recept-voorblad'!$A$89:$H$93,5,FALSE())</f>
+        <f>VLOOKUP("*Nagardo*",'Recept-voorblad'!$A$91:$H$93,5,FALSE())</f>
         <v/>
       </c>
       <c r="W36" s="1602" t="inlineStr">
@@ -25823,7 +25877,7 @@
       <c r="T46" s="1954" t="n"/>
       <c r="U46" s="1955" t="n"/>
       <c r="V46" s="1955">
-        <f>'Recept-voorblad'!$E$90*(V35/100*100)</f>
+        <f>'Recept-voorblad'!$E$92*(V35/100*100)</f>
         <v/>
       </c>
       <c r="W46" s="1954" t="inlineStr">
@@ -26030,7 +26084,7 @@
       <c r="T50" s="1602" t="n"/>
       <c r="U50" s="1602" t="n"/>
       <c r="V50" s="1763">
-        <f>VLOOKUP("*Nagardo*",'Recept-voorblad'!$A$89:$H$93,5,FALSE())</f>
+        <f>VLOOKUP("*Nagardo*",'Recept-voorblad'!$A$91:$H$93,5,FALSE())</f>
         <v/>
       </c>
       <c r="W50" s="1602" t="inlineStr">
@@ -26517,7 +26571,7 @@
       <c r="T60" s="1602" t="n"/>
       <c r="U60" s="1763" t="n"/>
       <c r="V60" s="1763">
-        <f>'Recept-voorblad'!$E$90*(V49/100*100)</f>
+        <f>'Recept-voorblad'!$E$92*(V49/100*100)</f>
         <v/>
       </c>
       <c r="W60" s="1602" t="inlineStr">

</xml_diff>